<commit_message>
Contar por fatura do cartão (26 a 25) e tratar (banri) como vale-alimentação
Gastos antes de 26/10/2026 são descartados. Painel e planilha agrupam por
ciclo da fatura e mostram o gasto no vale, com saldo quando o valor
mensal do vale for informado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U9H2bpPTgH33XhYCozzWVS
</commit_message>
<xml_diff>
--- a/planilha/Gastos_Casa.xlsx
+++ b/planilha/Gastos_Casa.xlsx
@@ -20,11 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="166" formatCode="&quot;R$&quot; #,##0.00;-&quot;R$&quot; #,##0.00;&quot;-&quot;"/>
-    <numFmt numFmtId="167" formatCode="mmm/yyyy"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="&quot;R$&quot; #,##0.00;-&quot;R$&quot; #,##0.00;&quot;-&quot;"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -123,37 +122,38 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -252,7 +252,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Total por mês</a:t>
+              <a:t>Total por fatura</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -346,7 +346,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Por categoria (mês mais recente com gastos)</a:t>
+              <a:t>Por categoria (fatura atual)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -416,7 +416,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Planejamento'!C19</f>
+              <f>'Planejamento'!C22</f>
             </strRef>
           </tx>
           <spPr>
@@ -426,12 +426,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Planejamento'!$A$20:$A$23</f>
+              <f>'Planejamento'!$A$23:$A$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Planejamento'!$C$20:$C$23</f>
+              <f>'Planejamento'!$C$23:$C$26</f>
             </numRef>
           </val>
         </ser>
@@ -476,7 +476,7 @@
   <commentList>
     <comment ref="A5" authorId="0" shapeId="0">
       <text>
-        <t>Primeiro mês do grupo (outubro/2026). Os seguintes são calculados.</t>
+        <t>Início da primeira fatura anotada (26/10/2026, fechamento dos cartões). As seguintes são calculadas.</t>
       </text>
     </comment>
   </commentList>
@@ -494,34 +494,54 @@
         <t>Edite: quanto a mais separar além da média.</t>
       </text>
     </comment>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Dia em que a fatura dos cartões fecha.</t>
+      </text>
+    </comment>
+    <comment ref="B6" authorId="0" shapeId="0">
+      <text>
+        <t>Preencham com o valor que cai no vale por mês para ver o saldo.</t>
+      </text>
+    </comment>
     <comment ref="B7" authorId="0" shapeId="0">
       <text>
-        <t>Se o grupo começou no meio do mês, conta a partir daí.</t>
+        <t>Fatura do gasto mais recente.</t>
       </text>
     </comment>
-    <comment ref="B12" authorId="0" shapeId="0">
+    <comment ref="B10" authorId="0" shapeId="0">
+      <text>
+        <t>Do dia 26 até o gasto mais recente.</t>
+      </text>
+    </comment>
+    <comment ref="B13" authorId="0" shapeId="0">
       <text>
         <t>Gasto até agora + média por dia × dias que faltam.</t>
       </text>
     </comment>
-    <comment ref="B13" authorId="0" shapeId="0">
-      <text>
-        <t>Até 3 meses antes do mês mais recente.</t>
-      </text>
-    </comment>
     <comment ref="B14" authorId="0" shapeId="0">
       <text>
-        <t>Sem meses completos ainda, usa a projeção do mês.</t>
+        <t>Até 3 faturas antes da atual, com gastos.</t>
       </text>
     </comment>
     <comment ref="B15" authorId="0" shapeId="0">
       <text>
-        <t>Soma da tabela ao lado.</t>
+        <t>Sem faturas anteriores ainda, usa a projeção da atual.</t>
       </text>
     </comment>
     <comment ref="B16" authorId="0" shapeId="0">
       <text>
-        <t>(Média mensal + fixos) × (1 + margem).</t>
+        <t>Soma da tabela ao lado.</t>
+      </text>
+    </comment>
+    <comment ref="B17" authorId="0" shapeId="0">
+      <text>
+        <t>(Média por fatura + fixos) × (1 + margem).</t>
+      </text>
+    </comment>
+    <comment ref="B18" authorId="0" shapeId="0">
+      <text>
+        <t>Compras marcadas com (banri).</t>
       </text>
     </comment>
   </commentList>
@@ -583,7 +603,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>28</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5040000" cy="2520000"/>
@@ -893,7 +913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -937,201 +957,73 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>Linhas amarelas estão sem valor e não entram nos totais.</t>
+          <t>Linhas amarelas estão sem valor e não entram nos totais. (banri) = Vale-alimentação.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Almoço Bruna</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Alimentação</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="n">
-        <v>31</v>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Crédito</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>Bruna</t>
-        </is>
-      </c>
+      <c r="A2" s="3" t="n"/>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="5" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Morango + agua vinha paulinho</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Alimentação</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Banrisul</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Bruna</t>
-        </is>
-      </c>
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Zaffari</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Alimentação</t>
-        </is>
-      </c>
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
       <c r="D4" s="5" t="n"/>
       <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Tassio</t>
-        </is>
-      </c>
+      <c r="F4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
-        <v>46312</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Ildo</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Outros</t>
-        </is>
-      </c>
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Tassio</t>
-        </is>
-      </c>
+      <c r="F5" s="4" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
-        <v>46312</v>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Pipoca redenção</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Lazer</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>15</v>
-      </c>
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="5" t="n"/>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Tassio</t>
-        </is>
-      </c>
+      <c r="F6" s="4" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
-        <v>46313</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Bets</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Outros</t>
-        </is>
-      </c>
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="4" t="n"/>
       <c r="D7" s="5" t="n"/>
       <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Tassio</t>
-        </is>
-      </c>
+      <c r="F7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
-        <v>46313</v>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Uber teatro</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Transporte</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>11.35</v>
-      </c>
+      <c r="A8" s="3" t="n"/>
+      <c r="B8" s="4" t="n"/>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="5" t="n"/>
       <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Tassio</t>
-        </is>
-      </c>
+      <c r="F8" s="4" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
-        <v>46313</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Zafari</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Alimentação</t>
-        </is>
-      </c>
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="n"/>
       <c r="D9" s="5" t="n"/>
       <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Tassio</t>
-        </is>
-      </c>
+      <c r="F9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -1469,70 +1361,6 @@
       <c r="E51" s="4" t="n"/>
       <c r="F51" s="4" t="n"/>
     </row>
-    <row r="52">
-      <c r="A52" s="3" t="n"/>
-      <c r="B52" s="4" t="n"/>
-      <c r="C52" s="4" t="n"/>
-      <c r="D52" s="5" t="n"/>
-      <c r="E52" s="4" t="n"/>
-      <c r="F52" s="4" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="3" t="n"/>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="5" t="n"/>
-      <c r="E53" s="4" t="n"/>
-      <c r="F53" s="4" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="3" t="n"/>
-      <c r="B54" s="4" t="n"/>
-      <c r="C54" s="4" t="n"/>
-      <c r="D54" s="5" t="n"/>
-      <c r="E54" s="4" t="n"/>
-      <c r="F54" s="4" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="n"/>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="5" t="n"/>
-      <c r="E55" s="4" t="n"/>
-      <c r="F55" s="4" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="n"/>
-      <c r="B56" s="4" t="n"/>
-      <c r="C56" s="4" t="n"/>
-      <c r="D56" s="5" t="n"/>
-      <c r="E56" s="4" t="n"/>
-      <c r="F56" s="4" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="n"/>
-      <c r="B57" s="4" t="n"/>
-      <c r="C57" s="4" t="n"/>
-      <c r="D57" s="5" t="n"/>
-      <c r="E57" s="4" t="n"/>
-      <c r="F57" s="4" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="3" t="n"/>
-      <c r="B58" s="4" t="n"/>
-      <c r="C58" s="4" t="n"/>
-      <c r="D58" s="5" t="n"/>
-      <c r="E58" s="4" t="n"/>
-      <c r="F58" s="4" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="n"/>
-      <c r="B59" s="4" t="n"/>
-      <c r="C59" s="4" t="n"/>
-      <c r="D59" s="5" t="n"/>
-      <c r="E59" s="4" t="n"/>
-      <c r="F59" s="4" t="n"/>
-    </row>
   </sheetData>
   <autoFilter ref="A1:F1001"/>
   <conditionalFormatting sqref="A2:F1001">
@@ -1540,9 +1368,12 @@
       <formula>AND($B2&lt;&gt;"",$D2="")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="C2:C1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Categoria" error="Escolha uma das categorias da lista." type="list">
       <formula1>"Alimentação,Casa/contas,Transporte,Saúde,Lazer,Outros"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Pagamento" error="Escolha uma das formas de pagamento da lista." type="list">
+      <formula1>"Crédito,Débito,Pix,Dinheiro,Vale-alimentação"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1558,11 +1389,12 @@
   <dimension ref="A1:S19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
@@ -1581,21 +1413,21 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Gastos Casa — resumo por mês</t>
+          <t>Gastos Casa — resumo por fatura</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Totais calculados a partir da aba Lançamentos. Itens sem valor contam só como pendentes.</t>
+          <t>Cada fatura vai do dia de fechamento (26) ao dia 25 seguinte. Itens sem valor contam só como pendentes.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Mês</t>
+          <t>Fatura (início)</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -1615,7 +1447,12 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>Vs. mês anterior</t>
+          <t>Vs. fatura anterior</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>No vale</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1674,7 +1511,7 @@
     </row>
     <row r="5">
       <c r="A5" s="9" t="n">
-        <v>46296</v>
+        <v>46321</v>
       </c>
       <c r="B5" s="5">
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1))</f>
@@ -1689,6 +1526,10 @@
         <v/>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
           <t>Alimentação</t>
@@ -1744,7 +1585,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11">
+      <c r="A6" s="3">
         <f>EDATE(A5,1)</f>
         <v/>
       </c>
@@ -1764,6 +1605,10 @@
         <f>IF(B6=0,"",B6-B5)</f>
         <v/>
       </c>
+      <c r="F6" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
           <t>Casa/contas</t>
@@ -1819,7 +1664,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11">
+      <c r="A7" s="3">
         <f>EDATE(A6,1)</f>
         <v/>
       </c>
@@ -1839,6 +1684,10 @@
         <f>IF(B7=0,"",B7-B6)</f>
         <v/>
       </c>
+      <c r="F7" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
           <t>Transporte</t>
@@ -1894,7 +1743,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11">
+      <c r="A8" s="3">
         <f>EDATE(A7,1)</f>
         <v/>
       </c>
@@ -1914,6 +1763,10 @@
         <f>IF(B8=0,"",B8-B7)</f>
         <v/>
       </c>
+      <c r="F8" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
           <t>Saúde</t>
@@ -1969,7 +1822,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11">
+      <c r="A9" s="3">
         <f>EDATE(A8,1)</f>
         <v/>
       </c>
@@ -1989,6 +1842,10 @@
         <f>IF(B9=0,"",B9-B8)</f>
         <v/>
       </c>
+      <c r="F9" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
           <t>Lazer</t>
@@ -2044,7 +1901,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11">
+      <c r="A10" s="3">
         <f>EDATE(A9,1)</f>
         <v/>
       </c>
@@ -2064,6 +1921,10 @@
         <f>IF(B10=0,"",B10-B9)</f>
         <v/>
       </c>
+      <c r="F10" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
           <t>Outros</t>
@@ -2119,7 +1980,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11">
+      <c r="A11" s="3">
         <f>EDATE(A10,1)</f>
         <v/>
       </c>
@@ -2139,62 +2000,66 @@
         <f>IF(B11=0,"",B11-B10)</f>
         <v/>
       </c>
-      <c r="G11" s="12" t="inlineStr">
+      <c r="F11" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="H11" s="13">
+      <c r="H11" s="12">
         <f>SUM(H5:H10)</f>
         <v/>
       </c>
-      <c r="I11" s="13">
+      <c r="I11" s="12">
         <f>SUM(I5:I10)</f>
         <v/>
       </c>
-      <c r="J11" s="13">
+      <c r="J11" s="12">
         <f>SUM(J5:J10)</f>
         <v/>
       </c>
-      <c r="K11" s="13">
+      <c r="K11" s="12">
         <f>SUM(K5:K10)</f>
         <v/>
       </c>
-      <c r="L11" s="13">
+      <c r="L11" s="12">
         <f>SUM(L5:L10)</f>
         <v/>
       </c>
-      <c r="M11" s="13">
+      <c r="M11" s="12">
         <f>SUM(M5:M10)</f>
         <v/>
       </c>
-      <c r="N11" s="13">
+      <c r="N11" s="12">
         <f>SUM(N5:N10)</f>
         <v/>
       </c>
-      <c r="O11" s="13">
+      <c r="O11" s="12">
         <f>SUM(O5:O10)</f>
         <v/>
       </c>
-      <c r="P11" s="13">
+      <c r="P11" s="12">
         <f>SUM(P5:P10)</f>
         <v/>
       </c>
-      <c r="Q11" s="13">
+      <c r="Q11" s="12">
         <f>SUM(Q5:Q10)</f>
         <v/>
       </c>
-      <c r="R11" s="13">
+      <c r="R11" s="12">
         <f>SUM(R5:R10)</f>
         <v/>
       </c>
-      <c r="S11" s="13">
+      <c r="S11" s="12">
         <f>SUM(S5:S10)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11">
+      <c r="A12" s="3">
         <f>EDATE(A11,1)</f>
         <v/>
       </c>
@@ -2214,9 +2079,13 @@
         <f>IF(B12=0,"",B12-B11)</f>
         <v/>
       </c>
+      <c r="F12" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="11">
+      <c r="A13" s="3">
         <f>EDATE(A12,1)</f>
         <v/>
       </c>
@@ -2236,18 +2105,22 @@
         <f>IF(B13=0,"",B13-B12)</f>
         <v/>
       </c>
+      <c r="F13" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Mês mais recente</t>
-        </is>
-      </c>
-      <c r="H13" s="14">
-        <f>DATE(YEAR(MAX(Lançamentos!$A$2:$A$1001)),MONTH(MAX(Lançamentos!$A$2:$A$1001)),1)</f>
+          <t>Fatura atual</t>
+        </is>
+      </c>
+      <c r="H13" s="13">
+        <f>Planejamento!$B$7</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11">
+      <c r="A14" s="3">
         <f>EDATE(A13,1)</f>
         <v/>
       </c>
@@ -2267,17 +2140,21 @@
         <f>IF(B14=0,"",B14-B13)</f>
         <v/>
       </c>
+      <c r="F14" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
       <c r="G14" s="10">
         <f>G5</f>
         <v/>
       </c>
-      <c r="H14" s="15">
+      <c r="H14" s="14">
         <f>INDEX($H5:$S5,MATCH($H$13,$H$4:$S$4,0))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11">
+      <c r="A15" s="3">
         <f>EDATE(A14,1)</f>
         <v/>
       </c>
@@ -2297,17 +2174,21 @@
         <f>IF(B15=0,"",B15-B14)</f>
         <v/>
       </c>
+      <c r="F15" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
       <c r="G15" s="10">
         <f>G6</f>
         <v/>
       </c>
-      <c r="H15" s="15">
+      <c r="H15" s="14">
         <f>INDEX($H6:$S6,MATCH($H$13,$H$4:$S$4,0))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11">
+      <c r="A16" s="3">
         <f>EDATE(A15,1)</f>
         <v/>
       </c>
@@ -2327,11 +2208,15 @@
         <f>IF(B16=0,"",B16-B15)</f>
         <v/>
       </c>
+      <c r="F16" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
       <c r="G16" s="10">
         <f>G7</f>
         <v/>
       </c>
-      <c r="H16" s="15">
+      <c r="H16" s="14">
         <f>INDEX($H7:$S7,MATCH($H$13,$H$4:$S$4,0))</f>
         <v/>
       </c>
@@ -2341,7 +2226,7 @@
         <f>G8</f>
         <v/>
       </c>
-      <c r="H17" s="15">
+      <c r="H17" s="14">
         <f>INDEX($H8:$S8,MATCH($H$13,$H$4:$S$4,0))</f>
         <v/>
       </c>
@@ -2351,7 +2236,7 @@
         <f>G9</f>
         <v/>
       </c>
-      <c r="H18" s="15">
+      <c r="H18" s="14">
         <f>INDEX($H9:$S9,MATCH($H$13,$H$4:$S$4,0))</f>
         <v/>
       </c>
@@ -2361,7 +2246,7 @@
         <f>G10</f>
         <v/>
       </c>
-      <c r="H19" s="15">
+      <c r="H19" s="14">
         <f>INDEX($H10:$S10,MATCH($H$13,$H$4:$S$4,0))</f>
         <v/>
       </c>
@@ -2379,7 +2264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2399,12 +2284,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quanto separar por mês no ritmo atual. Células amarelas são para vocês editarem.</t>
+          <t>Quanto separar por fatura no ritmo atual. Células amarelas são para vocês editarem.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="E3" s="16" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Gastos fixos mensais fora do grupo</t>
         </is>
@@ -2416,15 +2301,15 @@
           <t>Margem de segurança</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="16" t="n">
         <v>0.1</v>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>Valor por mês</t>
         </is>
@@ -2433,12 +2318,11 @@
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>Mês mais recente</t>
-        </is>
-      </c>
-      <c r="B5" s="11">
-        <f>DATE(YEAR(MAX(Lançamentos!$A$2:$A$1001)),MONTH(MAX(Lançamentos!$A$2:$A$1001)),1)</f>
-        <v/>
+          <t>Dia de fechamento da fatura</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="n">
+        <v>26</v>
       </c>
       <c r="E5" s="19" t="n"/>
       <c r="F5" s="20" t="n"/>
@@ -2446,24 +2330,21 @@
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>Gasto no mês mais recente</t>
-        </is>
-      </c>
-      <c r="B6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(B5,1))</f>
-        <v/>
-      </c>
+          <t>Vale-alimentação por mês</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="n"/>
       <c r="E6" s="19" t="n"/>
       <c r="F6" s="20" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>Primeiro dia com anotação no mês</t>
-        </is>
-      </c>
-      <c r="B7" s="21">
-        <f>IF(MIN(Lançamentos!$A$2:$A$1001)&gt;=B5,DAY(MIN(Lançamentos!$A$2:$A$1001)),1)</f>
+          <t>Fatura atual (início)</t>
+        </is>
+      </c>
+      <c r="B7" s="3">
+        <f>IF(COUNT(Lançamentos!$A$2:$A$1001)=0,Resumo!$A$5,DATE(YEAR(MAX(Lançamentos!$A$2:$A$1001)),MONTH(MAX(Lançamentos!$A$2:$A$1001))-IF(DAY(MAX(Lançamentos!$A$2:$A$1001))&lt;B5,1,0),B5))</f>
         <v/>
       </c>
       <c r="E7" s="19" t="n"/>
@@ -2472,11 +2353,11 @@
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Último dia com anotação</t>
-        </is>
-      </c>
-      <c r="B8" s="21">
-        <f>DAY(MAX(Lançamentos!$A$2:$A$1001))</f>
+          <t>Fatura atual (fim)</t>
+        </is>
+      </c>
+      <c r="B8" s="3">
+        <f>EDATE(B7,1)-1</f>
         <v/>
       </c>
       <c r="E8" s="19" t="n"/>
@@ -2485,11 +2366,11 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Dias com anotações</t>
-        </is>
-      </c>
-      <c r="B9" s="21">
-        <f>B8-B7+1</f>
+          <t>Gasto na fatura atual</t>
+        </is>
+      </c>
+      <c r="B9" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B7,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B8)</f>
         <v/>
       </c>
       <c r="E9" s="19" t="n"/>
@@ -2498,11 +2379,11 @@
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Dias no mês</t>
-        </is>
-      </c>
-      <c r="B10" s="21">
-        <f>DAY(EOMONTH(B5,0))</f>
+          <t>Dias com anotações</t>
+        </is>
+      </c>
+      <c r="B10" s="22">
+        <f>IF(COUNT(Lançamentos!$A$2:$A$1001)=0,0,MAX(Lançamentos!$A$2:$A$1001)-B7+1)</f>
         <v/>
       </c>
       <c r="E10" s="19" t="n"/>
@@ -2511,11 +2392,11 @@
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Média por dia</t>
-        </is>
-      </c>
-      <c r="B11" s="5">
-        <f>IF(B9=0,0,B6/B9)</f>
+          <t>Dias na fatura</t>
+        </is>
+      </c>
+      <c r="B11" s="22">
+        <f>B8-B7+1</f>
         <v/>
       </c>
       <c r="E11" s="19" t="n"/>
@@ -2524,11 +2405,11 @@
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Projeção do mês</t>
+          <t>Média por dia</t>
         </is>
       </c>
       <c r="B12" s="5">
-        <f>B6+B11*(B10-B8)</f>
+        <f>IF(B10=0,0,B9/B10)</f>
         <v/>
       </c>
       <c r="E12" s="19" t="n"/>
@@ -2537,11 +2418,11 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Meses completos anteriores usados</t>
-        </is>
-      </c>
-      <c r="B13" s="21">
-        <f>COUNTIFS(Resumo!$A$5:$A$16,"&gt;="&amp;EDATE(B5,-3),Resumo!$A$5:$A$16,"&lt;"&amp;B5,Resumo!$B$5:$B$16,"&gt;0")</f>
+          <t>Projeção da fatura</t>
+        </is>
+      </c>
+      <c r="B13" s="5">
+        <f>B9+B12*(B11-B10)</f>
         <v/>
       </c>
       <c r="E13" s="19" t="n"/>
@@ -2550,11 +2431,11 @@
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>Média mensal (gastos do grupo)</t>
-        </is>
-      </c>
-      <c r="B14" s="5">
-        <f>IF(B13=0,B12,AVERAGEIFS(Resumo!$B$5:$B$16,Resumo!$A$5:$A$16,"&gt;="&amp;EDATE(B5,-3),Resumo!$A$5:$A$16,"&lt;"&amp;B5,Resumo!$B$5:$B$16,"&gt;0"))</f>
+          <t>Faturas anteriores usadas</t>
+        </is>
+      </c>
+      <c r="B14" s="22">
+        <f>COUNTIFS(Resumo!$A$5:$A$16,"&gt;="&amp;EDATE(B7,-3),Resumo!$A$5:$A$16,"&lt;"&amp;B7,Resumo!$B$5:$B$16,"&gt;0")</f>
         <v/>
       </c>
       <c r="E14" s="19" t="n"/>
@@ -2563,117 +2444,96 @@
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>Gastos fixos fora do grupo</t>
+          <t>Média por fatura (gastos do grupo)</t>
         </is>
       </c>
       <c r="B15" s="5">
-        <f>SUM(F5:F24)</f>
+        <f>IF(B14=0,B13,AVERAGEIFS(Resumo!$B$5:$B$16,Resumo!$A$5:$A$16,"&gt;="&amp;EDATE(B7,-3),Resumo!$A$5:$A$16,"&lt;"&amp;B7,Resumo!$B$5:$B$16,"&gt;0"))</f>
         <v/>
       </c>
       <c r="E15" s="19" t="n"/>
       <c r="F15" s="20" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="inlineStr">
-        <is>
-          <t>Separar por mês</t>
-        </is>
-      </c>
-      <c r="B16" s="23">
-        <f>(B14+B15)*(1+B4)</f>
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Gastos fixos fora do grupo</t>
+        </is>
+      </c>
+      <c r="B16" s="5">
+        <f>SUM(F5:F24)</f>
         <v/>
       </c>
       <c r="E16" s="19" t="n"/>
       <c r="F16" s="20" t="n"/>
     </row>
     <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>Separar por fatura</t>
+        </is>
+      </c>
+      <c r="B17" s="24">
+        <f>(B15+B16)*(1+B4)</f>
+        <v/>
+      </c>
       <c r="E17" s="19" t="n"/>
       <c r="F17" s="20" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>Reserva por horizonte</t>
-        </is>
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Gasto no vale nesta fatura</t>
+        </is>
+      </c>
+      <c r="B18" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B7,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B8,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
       </c>
       <c r="E18" s="19" t="n"/>
       <c r="F18" s="20" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>Horizonte</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
-        <is>
-          <t>Sem margem</t>
-        </is>
-      </c>
-      <c r="C19" s="1" t="inlineStr">
-        <is>
-          <t>Com margem</t>
-        </is>
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Saldo do vale</t>
+        </is>
+      </c>
+      <c r="B19" s="5">
+        <f>IF(B6="","Preencha o valor do vale",B6-B18)</f>
+        <v/>
       </c>
       <c r="E19" s="19" t="n"/>
       <c r="F19" s="20" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>1 mês</t>
-        </is>
-      </c>
-      <c r="B20" s="5">
-        <f>(B$14+B$15)*D20</f>
-        <v/>
-      </c>
-      <c r="C20" s="5">
-        <f>B$16*D20</f>
-        <v/>
-      </c>
-      <c r="D20" s="24" t="n">
-        <v>1</v>
-      </c>
       <c r="E20" s="19" t="n"/>
       <c r="F20" s="20" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>3 meses</t>
-        </is>
-      </c>
-      <c r="B21" s="5">
-        <f>(B$14+B$15)*D21</f>
-        <v/>
-      </c>
-      <c r="C21" s="5">
-        <f>B$16*D21</f>
-        <v/>
-      </c>
-      <c r="D21" s="24" t="n">
-        <v>3</v>
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Reserva por horizonte</t>
+        </is>
       </c>
       <c r="E21" s="19" t="n"/>
       <c r="F21" s="20" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>6 meses</t>
-        </is>
-      </c>
-      <c r="B22" s="5">
-        <f>(B$14+B$15)*D22</f>
-        <v/>
-      </c>
-      <c r="C22" s="5">
-        <f>B$16*D22</f>
-        <v/>
-      </c>
-      <c r="D22" s="24" t="n">
-        <v>6</v>
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>Horizonte</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>Sem margem</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>Com margem</t>
+        </is>
       </c>
       <c r="E22" s="19" t="n"/>
       <c r="F22" s="20" t="n"/>
@@ -2681,36 +2541,88 @@
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>12 meses</t>
+          <t>1 fatura</t>
         </is>
       </c>
       <c r="B23" s="5">
-        <f>(B$14+B$15)*D23</f>
+        <f>(B$15+B$16)*D23</f>
         <v/>
       </c>
       <c r="C23" s="5">
-        <f>B$16*D23</f>
-        <v/>
-      </c>
-      <c r="D23" s="24" t="n">
-        <v>12</v>
+        <f>B$17*D23</f>
+        <v/>
+      </c>
+      <c r="D23" s="25" t="n">
+        <v>1</v>
       </c>
       <c r="E23" s="19" t="n"/>
       <c r="F23" s="20" t="n"/>
     </row>
     <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>3 faturas</t>
+        </is>
+      </c>
+      <c r="B24" s="5">
+        <f>(B$15+B$16)*D24</f>
+        <v/>
+      </c>
+      <c r="C24" s="5">
+        <f>B$17*D24</f>
+        <v/>
+      </c>
+      <c r="D24" s="25" t="n">
+        <v>3</v>
+      </c>
       <c r="E24" s="19" t="n"/>
       <c r="F24" s="20" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Estimativa fica mais confiável a cada mês completo anotado.</t>
-        </is>
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>6 faturas</t>
+        </is>
+      </c>
+      <c r="B25" s="5">
+        <f>(B$15+B$16)*D25</f>
+        <v/>
+      </c>
+      <c r="C25" s="5">
+        <f>B$17*D25</f>
+        <v/>
+      </c>
+      <c r="D25" s="25" t="n">
+        <v>6</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Preencham aqui aluguel, condomínio, plano de saúde etc. (ex.: Aluguel | 1.800,00).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>12 faturas</t>
+        </is>
+      </c>
+      <c r="B26" s="5">
+        <f>(B$15+B$16)*D26</f>
+        <v/>
+      </c>
+      <c r="C26" s="5">
+        <f>B$17*D26</f>
+        <v/>
+      </c>
+      <c r="D26" s="25" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Estimativa fica mais confiável a cada fatura completa anotada.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Separar Cartão, Vale e Conta; painel lê a planilha ao vivo
Crédito vai para a fatura do mês seguinte e o vale sai do saldo do vale,
então os dois deixam de ser somados. O planejamento usa só cartão + conta,
o vale ganha saldo projetado no dia 25 e o total da casa fica só como
referência. O painel passa a ler a aba Lançamentos pelo conector
Google Sheets.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U9H2bpPTgH33XhYCozzWVS
</commit_message>
<xml_diff>
--- a/planilha/Gastos_Casa.xlsx
+++ b/planilha/Gastos_Casa.xlsx
@@ -68,12 +68,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="001E6B52"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001E6B52"/>
       <sz val="12"/>
     </font>
     <font>
@@ -122,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -139,33 +139,48 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FCE8B2"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00BF1A1A"/>
+      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -252,7 +267,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Total por fatura</a:t>
+              <a:t>Cartão e conta por fatura (sai do bolso)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -283,6 +298,30 @@
           <val>
             <numRef>
               <f>'Resumo'!$B$5:$B$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Resumo'!D4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Resumo'!$A$5:$A$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Resumo'!$D$5:$D$16</f>
             </numRef>
           </val>
         </ser>
@@ -328,6 +367,9 @@
         <crossAx val="10"/>
       </valAx>
     </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -346,7 +388,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Por categoria (fatura atual)</a:t>
+              <a:t>Por categoria na fatura atual (todas as formas)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -365,12 +407,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Resumo'!$G$14:$G$19</f>
+              <f>'Resumo'!$K$14:$K$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Resumo'!$H$14:$H$19</f>
+              <f>'Resumo'!$L$14:$L$19</f>
             </numRef>
           </val>
         </ser>
@@ -401,7 +443,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Quanto juntar (com margem)</a:t>
+              <a:t>Quanto juntar para cartão + conta (com margem)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -416,7 +458,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Planejamento'!C22</f>
+              <f>'Planejamento'!C32</f>
             </strRef>
           </tx>
           <spPr>
@@ -426,12 +468,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Planejamento'!$A$23:$A$26</f>
+              <f>'Planejamento'!$A$33:$A$36</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Planejamento'!$C$23:$C$26</f>
+              <f>'Planejamento'!$C$33:$C$36</f>
             </numRef>
           </val>
         </ser>
@@ -501,47 +543,62 @@
     </comment>
     <comment ref="B6" authorId="0" shapeId="0">
       <text>
-        <t>Preencham com o valor que cai no vale por mês para ver o saldo.</t>
-      </text>
-    </comment>
-    <comment ref="B7" authorId="0" shapeId="0">
-      <text>
         <t>Fatura do gasto mais recente.</t>
       </text>
     </comment>
-    <comment ref="B10" authorId="0" shapeId="0">
+    <comment ref="B9" authorId="0" shapeId="0">
       <text>
         <t>Do dia 26 até o gasto mais recente.</t>
       </text>
     </comment>
-    <comment ref="B13" authorId="0" shapeId="0">
+    <comment ref="B11" authorId="0" shapeId="0">
+      <text>
+        <t>Vai para a fatura que vocês pagam no mês seguinte.</t>
+      </text>
+    </comment>
+    <comment ref="B15" authorId="0" shapeId="0">
       <text>
         <t>Gasto até agora + média por dia × dias que faltam.</t>
       </text>
     </comment>
-    <comment ref="B14" authorId="0" shapeId="0">
+    <comment ref="B16" authorId="0" shapeId="0">
       <text>
         <t>Até 3 faturas antes da atual, com gastos.</t>
       </text>
     </comment>
-    <comment ref="B15" authorId="0" shapeId="0">
+    <comment ref="B17" authorId="0" shapeId="0">
       <text>
         <t>Sem faturas anteriores ainda, usa a projeção da atual.</t>
       </text>
     </comment>
-    <comment ref="B16" authorId="0" shapeId="0">
+    <comment ref="B18" authorId="0" shapeId="0">
       <text>
         <t>Soma da tabela ao lado.</t>
       </text>
     </comment>
-    <comment ref="B17" authorId="0" shapeId="0">
+    <comment ref="B19" authorId="0" shapeId="0">
       <text>
-        <t>(Média por fatura + fixos) × (1 + margem).</t>
+        <t>(Média cartão + conta + fixos) × (1 + margem). O vale fica de fora.</t>
       </text>
     </comment>
-    <comment ref="B18" authorId="0" shapeId="0">
+    <comment ref="B22" authorId="0" shapeId="0">
+      <text>
+        <t>Valor que cai no vale-alimentação por mês.</t>
+      </text>
+    </comment>
+    <comment ref="B23" authorId="0" shapeId="0">
       <text>
         <t>Compras marcadas com (banri).</t>
+      </text>
+    </comment>
+    <comment ref="B26" authorId="0" shapeId="0">
+      <text>
+        <t>Valor do vale menos o gasto projetado no ritmo atual.</t>
+      </text>
+    </comment>
+    <comment ref="B29" authorId="0" shapeId="0">
+      <text>
+        <t>Cartão + vale + conta, só para referência.</t>
       </text>
     </comment>
   </commentList>
@@ -554,7 +611,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6480000" cy="2880000"/>
@@ -574,9 +631,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>10</col>
+      <col>7</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="2880000"/>
@@ -603,7 +660,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>28</row>
+      <row>38</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5040000" cy="2520000"/>
@@ -1368,6 +1425,11 @@
       <formula>AND($B2&lt;&gt;"",$D2="")</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E1001">
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>AND($B2&lt;&gt;"",$E2="")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="C2:C1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Categoria" error="Escolha uma das categorias da lista." type="list">
       <formula1>"Alimentação,Casa/contas,Transporte,Saúde,Lazer,Outros"</formula1>
@@ -1386,20 +1448,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S19"/>
+  <dimension ref="A1:W19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="3" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
@@ -1408,6 +1470,10 @@
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
     <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1420,7 +1486,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cada fatura vai do dia de fechamento (26) ao dia 25 seguinte. Itens sem valor contam só como pendentes.</t>
+          <t>Cada fatura vai do dia 26 ao dia 25. Cartão = crédito (paga no mês seguinte); Vale = sai do saldo do vale; Conta = Pix, débito e dinheiro.</t>
         </is>
       </c>
     </row>
@@ -1432,79 +1498,94 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Cartão</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
+          <t>Vale</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Conta</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Cartão + conta</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
           <t>Gastos com valor</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>Sem valor</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Vs. fatura anterior</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>No vale</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>Cartão + conta vs. anterior</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>Gasto total da casa</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="H4" s="8">
+      <c r="L4" s="8">
         <f>A5</f>
         <v/>
       </c>
-      <c r="I4" s="8">
+      <c r="M4" s="8">
         <f>A6</f>
         <v/>
       </c>
-      <c r="J4" s="8">
+      <c r="N4" s="8">
         <f>A7</f>
         <v/>
       </c>
-      <c r="K4" s="8">
+      <c r="O4" s="8">
         <f>A8</f>
         <v/>
       </c>
-      <c r="L4" s="8">
+      <c r="P4" s="8">
         <f>A9</f>
         <v/>
       </c>
-      <c r="M4" s="8">
+      <c r="Q4" s="8">
         <f>A10</f>
         <v/>
       </c>
-      <c r="N4" s="8">
+      <c r="R4" s="8">
         <f>A11</f>
         <v/>
       </c>
-      <c r="O4" s="8">
+      <c r="S4" s="8">
         <f>A12</f>
         <v/>
       </c>
-      <c r="P4" s="8">
+      <c r="T4" s="8">
         <f>A13</f>
         <v/>
       </c>
-      <c r="Q4" s="8">
+      <c r="U4" s="8">
         <f>A14</f>
         <v/>
       </c>
-      <c r="R4" s="8">
+      <c r="V4" s="8">
         <f>A15</f>
         <v/>
       </c>
-      <c r="S4" s="8">
+      <c r="W4" s="8">
         <f>A16</f>
         <v/>
       </c>
@@ -1514,73 +1595,85 @@
         <v>46321</v>
       </c>
       <c r="B5" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C5" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D5" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="E5" s="5">
+        <f>B5+D5</f>
+        <v/>
+      </c>
+      <c r="F5" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="G5" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <v/>
+      </c>
+      <c r="H5" s="5" t="inlineStr"/>
+      <c r="I5" s="10">
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1))</f>
         <v/>
       </c>
-      <c r="C5" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="D5" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$D$2:$D$1001,"")</f>
-        <v/>
-      </c>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="K5" s="11" t="inlineStr">
         <is>
           <t>Alimentação</t>
         </is>
       </c>
-      <c r="H5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;H$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(H$4,1),Lançamentos!$C$2:$C$1001,$G5)</f>
-        <v/>
-      </c>
-      <c r="I5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;I$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(I$4,1),Lançamentos!$C$2:$C$1001,$G5)</f>
-        <v/>
-      </c>
-      <c r="J5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;J$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(J$4,1),Lançamentos!$C$2:$C$1001,$G5)</f>
-        <v/>
-      </c>
-      <c r="K5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;K$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(K$4,1),Lançamentos!$C$2:$C$1001,$G5)</f>
-        <v/>
-      </c>
       <c r="L5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$G5)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
         <v/>
       </c>
       <c r="M5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$G5)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
         <v/>
       </c>
       <c r="N5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$G5)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
         <v/>
       </c>
       <c r="O5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$G5)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
         <v/>
       </c>
       <c r="P5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$G5)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
         <v/>
       </c>
       <c r="Q5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$G5)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
         <v/>
       </c>
       <c r="R5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$G5)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
         <v/>
       </c>
       <c r="S5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$G5)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
+        <v/>
+      </c>
+      <c r="T5" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;T$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(T$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
+        <v/>
+      </c>
+      <c r="U5" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;U$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(U$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
+        <v/>
+      </c>
+      <c r="V5" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;V$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(V$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
+        <v/>
+      </c>
+      <c r="W5" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;W$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(W$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
         <v/>
       </c>
     </row>
@@ -1590,76 +1683,88 @@
         <v/>
       </c>
       <c r="B6" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C6" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D6" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="E6" s="5">
+        <f>B6+D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="G6" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <v/>
+      </c>
+      <c r="H6" s="5">
+        <f>IF(E6=0,"",E6-E5)</f>
+        <v/>
+      </c>
+      <c r="I6" s="10">
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1))</f>
         <v/>
       </c>
-      <c r="C6" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="D6" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$D$2:$D$1001,"")</f>
-        <v/>
-      </c>
-      <c r="E6" s="5">
-        <f>IF(B6=0,"",B6-B5)</f>
-        <v/>
-      </c>
-      <c r="F6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="K6" s="11" t="inlineStr">
         <is>
           <t>Casa/contas</t>
         </is>
       </c>
-      <c r="H6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;H$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(H$4,1),Lançamentos!$C$2:$C$1001,$G6)</f>
-        <v/>
-      </c>
-      <c r="I6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;I$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(I$4,1),Lançamentos!$C$2:$C$1001,$G6)</f>
-        <v/>
-      </c>
-      <c r="J6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;J$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(J$4,1),Lançamentos!$C$2:$C$1001,$G6)</f>
-        <v/>
-      </c>
-      <c r="K6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;K$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(K$4,1),Lançamentos!$C$2:$C$1001,$G6)</f>
-        <v/>
-      </c>
       <c r="L6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$G6)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
         <v/>
       </c>
       <c r="M6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$G6)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
         <v/>
       </c>
       <c r="N6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$G6)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
         <v/>
       </c>
       <c r="O6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$G6)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
         <v/>
       </c>
       <c r="P6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$G6)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
         <v/>
       </c>
       <c r="Q6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$G6)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
         <v/>
       </c>
       <c r="R6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$G6)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
         <v/>
       </c>
       <c r="S6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$G6)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
+        <v/>
+      </c>
+      <c r="T6" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;T$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(T$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
+        <v/>
+      </c>
+      <c r="U6" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;U$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(U$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
+        <v/>
+      </c>
+      <c r="V6" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;V$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(V$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
+        <v/>
+      </c>
+      <c r="W6" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;W$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(W$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
         <v/>
       </c>
     </row>
@@ -1669,76 +1774,88 @@
         <v/>
       </c>
       <c r="B7" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C7" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D7" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="E7" s="5">
+        <f>B7+D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="G7" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <v/>
+      </c>
+      <c r="H7" s="5">
+        <f>IF(E7=0,"",E7-E6)</f>
+        <v/>
+      </c>
+      <c r="I7" s="10">
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1))</f>
         <v/>
       </c>
-      <c r="C7" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="D7" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$D$2:$D$1001,"")</f>
-        <v/>
-      </c>
-      <c r="E7" s="5">
-        <f>IF(B7=0,"",B7-B6)</f>
-        <v/>
-      </c>
-      <c r="F7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>Transporte</t>
         </is>
       </c>
-      <c r="H7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;H$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(H$4,1),Lançamentos!$C$2:$C$1001,$G7)</f>
-        <v/>
-      </c>
-      <c r="I7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;I$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(I$4,1),Lançamentos!$C$2:$C$1001,$G7)</f>
-        <v/>
-      </c>
-      <c r="J7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;J$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(J$4,1),Lançamentos!$C$2:$C$1001,$G7)</f>
-        <v/>
-      </c>
-      <c r="K7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;K$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(K$4,1),Lançamentos!$C$2:$C$1001,$G7)</f>
-        <v/>
-      </c>
       <c r="L7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$G7)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
         <v/>
       </c>
       <c r="M7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$G7)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
         <v/>
       </c>
       <c r="N7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$G7)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
         <v/>
       </c>
       <c r="O7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$G7)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
         <v/>
       </c>
       <c r="P7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$G7)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
         <v/>
       </c>
       <c r="Q7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$G7)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
         <v/>
       </c>
       <c r="R7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$G7)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
         <v/>
       </c>
       <c r="S7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$G7)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
+        <v/>
+      </c>
+      <c r="T7" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;T$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(T$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
+        <v/>
+      </c>
+      <c r="U7" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;U$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(U$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
+        <v/>
+      </c>
+      <c r="V7" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;V$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(V$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
+        <v/>
+      </c>
+      <c r="W7" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;W$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(W$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
         <v/>
       </c>
     </row>
@@ -1748,76 +1865,88 @@
         <v/>
       </c>
       <c r="B8" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C8" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D8" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="E8" s="5">
+        <f>B8+D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="G8" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <v/>
+      </c>
+      <c r="H8" s="5">
+        <f>IF(E8=0,"",E8-E7)</f>
+        <v/>
+      </c>
+      <c r="I8" s="10">
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1))</f>
         <v/>
       </c>
-      <c r="C8" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="D8" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$D$2:$D$1001,"")</f>
-        <v/>
-      </c>
-      <c r="E8" s="5">
-        <f>IF(B8=0,"",B8-B7)</f>
-        <v/>
-      </c>
-      <c r="F8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="K8" s="11" t="inlineStr">
         <is>
           <t>Saúde</t>
         </is>
       </c>
-      <c r="H8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;H$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(H$4,1),Lançamentos!$C$2:$C$1001,$G8)</f>
-        <v/>
-      </c>
-      <c r="I8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;I$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(I$4,1),Lançamentos!$C$2:$C$1001,$G8)</f>
-        <v/>
-      </c>
-      <c r="J8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;J$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(J$4,1),Lançamentos!$C$2:$C$1001,$G8)</f>
-        <v/>
-      </c>
-      <c r="K8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;K$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(K$4,1),Lançamentos!$C$2:$C$1001,$G8)</f>
-        <v/>
-      </c>
       <c r="L8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$G8)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
         <v/>
       </c>
       <c r="M8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$G8)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
         <v/>
       </c>
       <c r="N8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$G8)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
         <v/>
       </c>
       <c r="O8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$G8)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
         <v/>
       </c>
       <c r="P8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$G8)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
         <v/>
       </c>
       <c r="Q8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$G8)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
         <v/>
       </c>
       <c r="R8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$G8)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
         <v/>
       </c>
       <c r="S8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$G8)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
+        <v/>
+      </c>
+      <c r="T8" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;T$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(T$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
+        <v/>
+      </c>
+      <c r="U8" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;U$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(U$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
+        <v/>
+      </c>
+      <c r="V8" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;V$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(V$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
+        <v/>
+      </c>
+      <c r="W8" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;W$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(W$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
         <v/>
       </c>
     </row>
@@ -1827,76 +1956,88 @@
         <v/>
       </c>
       <c r="B9" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C9" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D9" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="E9" s="5">
+        <f>B9+D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="G9" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <v/>
+      </c>
+      <c r="H9" s="5">
+        <f>IF(E9=0,"",E9-E8)</f>
+        <v/>
+      </c>
+      <c r="I9" s="10">
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1))</f>
         <v/>
       </c>
-      <c r="C9" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="D9" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$D$2:$D$1001,"")</f>
-        <v/>
-      </c>
-      <c r="E9" s="5">
-        <f>IF(B9=0,"",B9-B8)</f>
-        <v/>
-      </c>
-      <c r="F9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="K9" s="11" t="inlineStr">
         <is>
           <t>Lazer</t>
         </is>
       </c>
-      <c r="H9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;H$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(H$4,1),Lançamentos!$C$2:$C$1001,$G9)</f>
-        <v/>
-      </c>
-      <c r="I9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;I$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(I$4,1),Lançamentos!$C$2:$C$1001,$G9)</f>
-        <v/>
-      </c>
-      <c r="J9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;J$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(J$4,1),Lançamentos!$C$2:$C$1001,$G9)</f>
-        <v/>
-      </c>
-      <c r="K9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;K$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(K$4,1),Lançamentos!$C$2:$C$1001,$G9)</f>
-        <v/>
-      </c>
       <c r="L9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$G9)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
         <v/>
       </c>
       <c r="M9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$G9)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
         <v/>
       </c>
       <c r="N9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$G9)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
         <v/>
       </c>
       <c r="O9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$G9)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
         <v/>
       </c>
       <c r="P9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$G9)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
         <v/>
       </c>
       <c r="Q9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$G9)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
         <v/>
       </c>
       <c r="R9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$G9)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
         <v/>
       </c>
       <c r="S9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$G9)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
+        <v/>
+      </c>
+      <c r="T9" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;T$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(T$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
+        <v/>
+      </c>
+      <c r="U9" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;U$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(U$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
+        <v/>
+      </c>
+      <c r="V9" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;V$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(V$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
+        <v/>
+      </c>
+      <c r="W9" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;W$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(W$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
         <v/>
       </c>
     </row>
@@ -1906,76 +2047,88 @@
         <v/>
       </c>
       <c r="B10" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C10" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D10" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="E10" s="5">
+        <f>B10+D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="G10" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <v/>
+      </c>
+      <c r="H10" s="5">
+        <f>IF(E10=0,"",E10-E9)</f>
+        <v/>
+      </c>
+      <c r="I10" s="10">
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1))</f>
         <v/>
       </c>
-      <c r="C10" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="D10" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$D$2:$D$1001,"")</f>
-        <v/>
-      </c>
-      <c r="E10" s="5">
-        <f>IF(B10=0,"",B10-B9)</f>
-        <v/>
-      </c>
-      <c r="F10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="K10" s="11" t="inlineStr">
         <is>
           <t>Outros</t>
         </is>
       </c>
-      <c r="H10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;H$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(H$4,1),Lançamentos!$C$2:$C$1001,$G10)</f>
-        <v/>
-      </c>
-      <c r="I10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;I$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(I$4,1),Lançamentos!$C$2:$C$1001,$G10)</f>
-        <v/>
-      </c>
-      <c r="J10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;J$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(J$4,1),Lançamentos!$C$2:$C$1001,$G10)</f>
-        <v/>
-      </c>
-      <c r="K10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;K$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(K$4,1),Lançamentos!$C$2:$C$1001,$G10)</f>
-        <v/>
-      </c>
       <c r="L10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$G10)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
         <v/>
       </c>
       <c r="M10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$G10)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
         <v/>
       </c>
       <c r="N10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$G10)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
         <v/>
       </c>
       <c r="O10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$G10)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
         <v/>
       </c>
       <c r="P10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$G10)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
         <v/>
       </c>
       <c r="Q10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$G10)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
         <v/>
       </c>
       <c r="R10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$G10)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
         <v/>
       </c>
       <c r="S10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$G10)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
+        <v/>
+      </c>
+      <c r="T10" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;T$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(T$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
+        <v/>
+      </c>
+      <c r="U10" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;U$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(U$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
+        <v/>
+      </c>
+      <c r="V10" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;V$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(V$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
+        <v/>
+      </c>
+      <c r="W10" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;W$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(W$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
         <v/>
       </c>
     </row>
@@ -1985,76 +2138,88 @@
         <v/>
       </c>
       <c r="B11" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C11" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D11" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="E11" s="5">
+        <f>B11+D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="G11" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <v/>
+      </c>
+      <c r="H11" s="5">
+        <f>IF(E11=0,"",E11-E10)</f>
+        <v/>
+      </c>
+      <c r="I11" s="10">
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1))</f>
         <v/>
       </c>
-      <c r="C11" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="D11" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$D$2:$D$1001,"")</f>
-        <v/>
-      </c>
-      <c r="E11" s="5">
-        <f>IF(B11=0,"",B11-B10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="G11" s="11" t="inlineStr">
+      <c r="K11" s="12" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="H11" s="12">
-        <f>SUM(H5:H10)</f>
-        <v/>
-      </c>
-      <c r="I11" s="12">
-        <f>SUM(I5:I10)</f>
-        <v/>
-      </c>
-      <c r="J11" s="12">
-        <f>SUM(J5:J10)</f>
-        <v/>
-      </c>
-      <c r="K11" s="12">
-        <f>SUM(K5:K10)</f>
-        <v/>
-      </c>
-      <c r="L11" s="12">
+      <c r="L11" s="13">
         <f>SUM(L5:L10)</f>
         <v/>
       </c>
-      <c r="M11" s="12">
+      <c r="M11" s="13">
         <f>SUM(M5:M10)</f>
         <v/>
       </c>
-      <c r="N11" s="12">
+      <c r="N11" s="13">
         <f>SUM(N5:N10)</f>
         <v/>
       </c>
-      <c r="O11" s="12">
+      <c r="O11" s="13">
         <f>SUM(O5:O10)</f>
         <v/>
       </c>
-      <c r="P11" s="12">
+      <c r="P11" s="13">
         <f>SUM(P5:P10)</f>
         <v/>
       </c>
-      <c r="Q11" s="12">
+      <c r="Q11" s="13">
         <f>SUM(Q5:Q10)</f>
         <v/>
       </c>
-      <c r="R11" s="12">
+      <c r="R11" s="13">
         <f>SUM(R5:R10)</f>
         <v/>
       </c>
-      <c r="S11" s="12">
+      <c r="S11" s="13">
         <f>SUM(S5:S10)</f>
+        <v/>
+      </c>
+      <c r="T11" s="13">
+        <f>SUM(T5:T10)</f>
+        <v/>
+      </c>
+      <c r="U11" s="13">
+        <f>SUM(U5:U10)</f>
+        <v/>
+      </c>
+      <c r="V11" s="13">
+        <f>SUM(V5:V10)</f>
+        <v/>
+      </c>
+      <c r="W11" s="13">
+        <f>SUM(W5:W10)</f>
         <v/>
       </c>
     </row>
@@ -2064,23 +2229,35 @@
         <v/>
       </c>
       <c r="B12" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C12" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D12" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="E12" s="5">
+        <f>B12+D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="G12" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <v/>
+      </c>
+      <c r="H12" s="5">
+        <f>IF(E12=0,"",E12-E11)</f>
+        <v/>
+      </c>
+      <c r="I12" s="10">
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1))</f>
-        <v/>
-      </c>
-      <c r="C12" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="D12" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$D$2:$D$1001,"")</f>
-        <v/>
-      </c>
-      <c r="E12" s="5">
-        <f>IF(B12=0,"",B12-B11)</f>
-        <v/>
-      </c>
-      <c r="F12" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
         <v/>
       </c>
     </row>
@@ -2090,32 +2267,44 @@
         <v/>
       </c>
       <c r="B13" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C13" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D13" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="E13" s="5">
+        <f>B13+D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="G13" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <v/>
+      </c>
+      <c r="H13" s="5">
+        <f>IF(E13=0,"",E13-E12)</f>
+        <v/>
+      </c>
+      <c r="I13" s="10">
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1))</f>
         <v/>
       </c>
-      <c r="C13" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="D13" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$D$2:$D$1001,"")</f>
-        <v/>
-      </c>
-      <c r="E13" s="5">
-        <f>IF(B13=0,"",B13-B12)</f>
-        <v/>
-      </c>
-      <c r="F13" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Fatura atual</t>
         </is>
       </c>
-      <c r="H13" s="13">
-        <f>Planejamento!$B$7</f>
+      <c r="L13" s="14">
+        <f>Planejamento!$B$6</f>
         <v/>
       </c>
     </row>
@@ -2125,31 +2314,43 @@
         <v/>
       </c>
       <c r="B14" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C14" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D14" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="E14" s="5">
+        <f>B14+D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="G14" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <v/>
+      </c>
+      <c r="H14" s="5">
+        <f>IF(E14=0,"",E14-E13)</f>
+        <v/>
+      </c>
+      <c r="I14" s="10">
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1))</f>
         <v/>
       </c>
-      <c r="C14" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="D14" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$D$2:$D$1001,"")</f>
-        <v/>
-      </c>
-      <c r="E14" s="5">
-        <f>IF(B14=0,"",B14-B13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="G14" s="10">
-        <f>G5</f>
-        <v/>
-      </c>
-      <c r="H14" s="14">
-        <f>INDEX($H5:$S5,MATCH($H$13,$H$4:$S$4,0))</f>
+      <c r="K14" s="11">
+        <f>K5</f>
+        <v/>
+      </c>
+      <c r="L14" s="15">
+        <f>INDEX($L5:$W5,MATCH($L$13,$L$4:$W$4,0))</f>
         <v/>
       </c>
     </row>
@@ -2159,31 +2360,43 @@
         <v/>
       </c>
       <c r="B15" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C15" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D15" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="E15" s="5">
+        <f>B15+D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="G15" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <v/>
+      </c>
+      <c r="H15" s="5">
+        <f>IF(E15=0,"",E15-E14)</f>
+        <v/>
+      </c>
+      <c r="I15" s="10">
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1))</f>
         <v/>
       </c>
-      <c r="C15" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="D15" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$D$2:$D$1001,"")</f>
-        <v/>
-      </c>
-      <c r="E15" s="5">
-        <f>IF(B15=0,"",B15-B14)</f>
-        <v/>
-      </c>
-      <c r="F15" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="G15" s="10">
-        <f>G6</f>
-        <v/>
-      </c>
-      <c r="H15" s="14">
-        <f>INDEX($H6:$S6,MATCH($H$13,$H$4:$S$4,0))</f>
+      <c r="K15" s="11">
+        <f>K6</f>
+        <v/>
+      </c>
+      <c r="L15" s="15">
+        <f>INDEX($L6:$W6,MATCH($L$13,$L$4:$W$4,0))</f>
         <v/>
       </c>
     </row>
@@ -2193,61 +2406,73 @@
         <v/>
       </c>
       <c r="B16" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C16" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D16" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="E16" s="5">
+        <f>B16+D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="G16" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <v/>
+      </c>
+      <c r="H16" s="5">
+        <f>IF(E16=0,"",E16-E15)</f>
+        <v/>
+      </c>
+      <c r="I16" s="10">
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1))</f>
         <v/>
       </c>
-      <c r="C16" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="D16" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$D$2:$D$1001,"")</f>
-        <v/>
-      </c>
-      <c r="E16" s="5">
-        <f>IF(B16=0,"",B16-B15)</f>
-        <v/>
-      </c>
-      <c r="F16" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="G16" s="10">
-        <f>G7</f>
-        <v/>
-      </c>
-      <c r="H16" s="14">
-        <f>INDEX($H7:$S7,MATCH($H$13,$H$4:$S$4,0))</f>
+      <c r="K16" s="11">
+        <f>K7</f>
+        <v/>
+      </c>
+      <c r="L16" s="15">
+        <f>INDEX($L7:$W7,MATCH($L$13,$L$4:$W$4,0))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="G17" s="10">
-        <f>G8</f>
-        <v/>
-      </c>
-      <c r="H17" s="14">
-        <f>INDEX($H8:$S8,MATCH($H$13,$H$4:$S$4,0))</f>
+      <c r="K17" s="11">
+        <f>K8</f>
+        <v/>
+      </c>
+      <c r="L17" s="15">
+        <f>INDEX($L8:$W8,MATCH($L$13,$L$4:$W$4,0))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="G18" s="10">
-        <f>G9</f>
-        <v/>
-      </c>
-      <c r="H18" s="14">
-        <f>INDEX($H9:$S9,MATCH($H$13,$H$4:$S$4,0))</f>
+      <c r="K18" s="11">
+        <f>K9</f>
+        <v/>
+      </c>
+      <c r="L18" s="15">
+        <f>INDEX($L9:$W9,MATCH($L$13,$L$4:$W$4,0))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="G19" s="10">
-        <f>G10</f>
-        <v/>
-      </c>
-      <c r="H19" s="14">
-        <f>INDEX($H10:$S10,MATCH($H$13,$H$4:$S$4,0))</f>
+      <c r="K19" s="11">
+        <f>K10</f>
+        <v/>
+      </c>
+      <c r="L19" s="15">
+        <f>INDEX($L10:$W10,MATCH($L$13,$L$4:$W$4,0))</f>
         <v/>
       </c>
     </row>
@@ -2264,12 +2489,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
@@ -2284,349 +2509,436 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quanto separar por fatura no ritmo atual. Células amarelas são para vocês editarem.</t>
+          <t>Cartão e conta saem do bolso; o vale é descontado do saldo do vale. Células amarelas são para vocês editarem.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="E3" s="15" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>Gastos fixos mensais fora do grupo</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Margem de segurança</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <v>0.1</v>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>Valor por mês</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Dia de fechamento da fatura</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="19" t="n">
         <v>26</v>
       </c>
-      <c r="E5" s="19" t="n"/>
-      <c r="F5" s="20" t="n"/>
+      <c r="E5" s="20" t="n"/>
+      <c r="F5" s="21" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>Vale-alimentação por mês</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="n"/>
-      <c r="E6" s="19" t="n"/>
-      <c r="F6" s="20" t="n"/>
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Fatura atual (início)</t>
+        </is>
+      </c>
+      <c r="B6" s="3">
+        <f>IF(COUNT(Lançamentos!$A$2:$A$1001)=0,Resumo!$A$5,DATE(YEAR(MAX(Lançamentos!$A$2:$A$1001)),MONTH(MAX(Lançamentos!$A$2:$A$1001))-IF(DAY(MAX(Lançamentos!$A$2:$A$1001))&lt;B5,1,0),B5))</f>
+        <v/>
+      </c>
+      <c r="E6" s="20" t="n"/>
+      <c r="F6" s="21" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>Fatura atual (início)</t>
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Fatura atual (fim)</t>
         </is>
       </c>
       <c r="B7" s="3">
-        <f>IF(COUNT(Lançamentos!$A$2:$A$1001)=0,Resumo!$A$5,DATE(YEAR(MAX(Lançamentos!$A$2:$A$1001)),MONTH(MAX(Lançamentos!$A$2:$A$1001))-IF(DAY(MAX(Lançamentos!$A$2:$A$1001))&lt;B5,1,0),B5))</f>
-        <v/>
-      </c>
-      <c r="E7" s="19" t="n"/>
-      <c r="F7" s="20" t="n"/>
+        <f>EDATE(B6,1)-1</f>
+        <v/>
+      </c>
+      <c r="E7" s="20" t="n"/>
+      <c r="F7" s="21" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>Fatura atual (fim)</t>
-        </is>
-      </c>
-      <c r="B8" s="3">
-        <f>EDATE(B7,1)-1</f>
-        <v/>
-      </c>
-      <c r="E8" s="19" t="n"/>
-      <c r="F8" s="20" t="n"/>
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Dias na fatura</t>
+        </is>
+      </c>
+      <c r="B8" s="22">
+        <f>B7-B6+1</f>
+        <v/>
+      </c>
+      <c r="E8" s="20" t="n"/>
+      <c r="F8" s="21" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>Gasto na fatura atual</t>
-        </is>
-      </c>
-      <c r="B9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B7,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="19" t="n"/>
-      <c r="F9" s="20" t="n"/>
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Dias com anotações</t>
+        </is>
+      </c>
+      <c r="B9" s="22">
+        <f>IF(COUNT(Lançamentos!$A$2:$A$1001)=0,0,MAX(Lançamentos!$A$2:$A$1001)-B6+1)</f>
+        <v/>
+      </c>
+      <c r="E9" s="20" t="n"/>
+      <c r="F9" s="21" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>Dias com anotações</t>
-        </is>
-      </c>
-      <c r="B10" s="22">
-        <f>IF(COUNT(Lançamentos!$A$2:$A$1001)=0,0,MAX(Lançamentos!$A$2:$A$1001)-B7+1)</f>
-        <v/>
-      </c>
-      <c r="E10" s="19" t="n"/>
-      <c r="F10" s="20" t="n"/>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Fatura do cartão + conta (sai do bolso)</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="n"/>
+      <c r="F10" s="21" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>Dias na fatura</t>
-        </is>
-      </c>
-      <c r="B11" s="22">
-        <f>B8-B7+1</f>
-        <v/>
-      </c>
-      <c r="E11" s="19" t="n"/>
-      <c r="F11" s="20" t="n"/>
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Cartão (crédito) nesta fatura</t>
+        </is>
+      </c>
+      <c r="B11" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B7,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="E11" s="20" t="n"/>
+      <c r="F11" s="21" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Conta (Pix, débito, dinheiro)</t>
+        </is>
+      </c>
+      <c r="B12" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B7,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B7,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B7,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="E12" s="20" t="n"/>
+      <c r="F12" s="21" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Cartão + conta</t>
+        </is>
+      </c>
+      <c r="B13" s="5">
+        <f>B11+B12</f>
+        <v/>
+      </c>
+      <c r="E13" s="20" t="n"/>
+      <c r="F13" s="21" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Média por dia</t>
         </is>
       </c>
-      <c r="B12" s="5">
-        <f>IF(B10=0,0,B9/B10)</f>
-        <v/>
-      </c>
-      <c r="E12" s="19" t="n"/>
-      <c r="F12" s="20" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>Projeção da fatura</t>
-        </is>
-      </c>
-      <c r="B13" s="5">
-        <f>B9+B12*(B11-B10)</f>
-        <v/>
-      </c>
-      <c r="E13" s="19" t="n"/>
-      <c r="F13" s="20" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="B14" s="5">
+        <f>IF(B9=0,0,B13/B9)</f>
+        <v/>
+      </c>
+      <c r="E14" s="20" t="n"/>
+      <c r="F14" s="21" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Projeção até o dia 25</t>
+        </is>
+      </c>
+      <c r="B15" s="5">
+        <f>B13+B14*(B8-B9)</f>
+        <v/>
+      </c>
+      <c r="E15" s="20" t="n"/>
+      <c r="F15" s="21" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Faturas anteriores usadas</t>
         </is>
       </c>
-      <c r="B14" s="22">
-        <f>COUNTIFS(Resumo!$A$5:$A$16,"&gt;="&amp;EDATE(B7,-3),Resumo!$A$5:$A$16,"&lt;"&amp;B7,Resumo!$B$5:$B$16,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="E14" s="19" t="n"/>
-      <c r="F14" s="20" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>Média por fatura (gastos do grupo)</t>
-        </is>
-      </c>
-      <c r="B15" s="5">
-        <f>IF(B14=0,B13,AVERAGEIFS(Resumo!$B$5:$B$16,Resumo!$A$5:$A$16,"&gt;="&amp;EDATE(B7,-3),Resumo!$A$5:$A$16,"&lt;"&amp;B7,Resumo!$B$5:$B$16,"&gt;0"))</f>
-        <v/>
-      </c>
-      <c r="E15" s="19" t="n"/>
-      <c r="F15" s="20" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="B16" s="22">
+        <f>COUNTIFS(Resumo!$A$5:$A$16,"&gt;="&amp;EDATE(B6,-3),Resumo!$A$5:$A$16,"&lt;"&amp;B6,Resumo!$E$5:$E$16,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="E16" s="20" t="n"/>
+      <c r="F16" s="21" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Média por fatura (cartão + conta)</t>
+        </is>
+      </c>
+      <c r="B17" s="5">
+        <f>IF(B16=0,B15,AVERAGEIFS(Resumo!$E$5:$E$16,Resumo!$A$5:$A$16,"&gt;="&amp;EDATE(B6,-3),Resumo!$A$5:$A$16,"&lt;"&amp;B6,Resumo!$E$5:$E$16,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="E17" s="20" t="n"/>
+      <c r="F17" s="21" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>Gastos fixos fora do grupo</t>
         </is>
       </c>
-      <c r="B16" s="5">
+      <c r="B18" s="5">
         <f>SUM(F5:F24)</f>
         <v/>
       </c>
-      <c r="E16" s="19" t="n"/>
-      <c r="F16" s="20" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="E18" s="20" t="n"/>
+      <c r="F18" s="21" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>Separar por fatura</t>
         </is>
       </c>
-      <c r="B17" s="24">
-        <f>(B15+B16)*(1+B4)</f>
-        <v/>
-      </c>
-      <c r="E17" s="19" t="n"/>
-      <c r="F17" s="20" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="B19" s="24">
+        <f>(B17+B18)*(1+B4)</f>
+        <v/>
+      </c>
+      <c r="E19" s="20" t="n"/>
+      <c r="F19" s="21" t="n"/>
+    </row>
+    <row r="20">
+      <c r="E20" s="20" t="n"/>
+      <c r="F20" s="21" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>Vale-alimentação (sai do saldo do vale)</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="n"/>
+      <c r="F21" s="21" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Vale por mês</t>
+        </is>
+      </c>
+      <c r="B22" s="25" t="n">
+        <v>2643.77</v>
+      </c>
+      <c r="E22" s="20" t="n"/>
+      <c r="F22" s="21" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Gasto no vale nesta fatura</t>
         </is>
       </c>
-      <c r="B18" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B7,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B8,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="E18" s="19" t="n"/>
-      <c r="F18" s="20" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>Saldo do vale</t>
-        </is>
-      </c>
-      <c r="B19" s="5">
-        <f>IF(B6="","Preencha o valor do vale",B6-B18)</f>
-        <v/>
-      </c>
-      <c r="E19" s="19" t="n"/>
-      <c r="F19" s="20" t="n"/>
-    </row>
-    <row r="20">
-      <c r="E20" s="19" t="n"/>
-      <c r="F20" s="20" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>Reserva por horizonte</t>
-        </is>
-      </c>
-      <c r="E21" s="19" t="n"/>
-      <c r="F21" s="20" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+      <c r="B23" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B7,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="E23" s="20" t="n"/>
+      <c r="F23" s="21" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>Saldo atual do vale</t>
+        </is>
+      </c>
+      <c r="B24" s="5">
+        <f>IF(B22="","Preencha o valor do vale",B22-B23)</f>
+        <v/>
+      </c>
+      <c r="E24" s="20" t="n"/>
+      <c r="F24" s="21" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>Média por dia no vale</t>
+        </is>
+      </c>
+      <c r="B25" s="5">
+        <f>IF(B9=0,0,B23/B9)</f>
+        <v/>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Preencham aqui aluguel, condomínio, plano de saúde etc. (ex.: Aluguel | 1.800,00).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>Saldo projetado no dia 25</t>
+        </is>
+      </c>
+      <c r="B26" s="5">
+        <f>IF(B22="","",B22-(B23+B25*(B8-B9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Situação do vale</t>
+        </is>
+      </c>
+      <c r="B27" s="26">
+        <f>IF(B22="","",IF(B26&lt;0,"Atenção: no ritmo atual o vale acaba antes do dia 25; faltam cerca de R$ "&amp;ROUND(-B26,0)&amp;", que vão cair no cartão ou na conta.","Dentro do saldo do vale"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Gasto total da casa nesta fatura (referência)</t>
+        </is>
+      </c>
+      <c r="B29" s="10">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>Reserva por horizonte (cartão + conta)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>Horizonte</t>
         </is>
       </c>
-      <c r="B22" s="1" t="inlineStr">
+      <c r="B32" s="1" t="inlineStr">
         <is>
           <t>Sem margem</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C32" s="1" t="inlineStr">
         <is>
           <t>Com margem</t>
         </is>
       </c>
-      <c r="E22" s="19" t="n"/>
-      <c r="F22" s="20" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>1 fatura</t>
         </is>
       </c>
-      <c r="B23" s="5">
-        <f>(B$15+B$16)*D23</f>
-        <v/>
-      </c>
-      <c r="C23" s="5">
-        <f>B$17*D23</f>
-        <v/>
-      </c>
-      <c r="D23" s="25" t="n">
+      <c r="B33" s="5">
+        <f>(B$17+B$18)*D33</f>
+        <v/>
+      </c>
+      <c r="C33" s="5">
+        <f>B$19*D33</f>
+        <v/>
+      </c>
+      <c r="D33" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="19" t="n"/>
-      <c r="F23" s="20" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>3 faturas</t>
         </is>
       </c>
-      <c r="B24" s="5">
-        <f>(B$15+B$16)*D24</f>
-        <v/>
-      </c>
-      <c r="C24" s="5">
-        <f>B$17*D24</f>
-        <v/>
-      </c>
-      <c r="D24" s="25" t="n">
+      <c r="B34" s="5">
+        <f>(B$17+B$18)*D34</f>
+        <v/>
+      </c>
+      <c r="C34" s="5">
+        <f>B$19*D34</f>
+        <v/>
+      </c>
+      <c r="D34" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="E24" s="19" t="n"/>
-      <c r="F24" s="20" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="10" t="inlineStr">
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>6 faturas</t>
         </is>
       </c>
-      <c r="B25" s="5">
-        <f>(B$15+B$16)*D25</f>
-        <v/>
-      </c>
-      <c r="C25" s="5">
-        <f>B$17*D25</f>
-        <v/>
-      </c>
-      <c r="D25" s="25" t="n">
+      <c r="B35" s="5">
+        <f>(B$17+B$18)*D35</f>
+        <v/>
+      </c>
+      <c r="C35" s="5">
+        <f>B$19*D35</f>
+        <v/>
+      </c>
+      <c r="D35" s="27" t="n">
         <v>6</v>
       </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Preencham aqui aluguel, condomínio, plano de saúde etc. (ex.: Aluguel | 1.800,00).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t>12 faturas</t>
         </is>
       </c>
-      <c r="B26" s="5">
-        <f>(B$15+B$16)*D26</f>
-        <v/>
-      </c>
-      <c r="C26" s="5">
-        <f>B$17*D26</f>
-        <v/>
-      </c>
-      <c r="D26" s="25" t="n">
+      <c r="B36" s="5">
+        <f>(B$17+B$18)*D36</f>
+        <v/>
+      </c>
+      <c r="C36" s="5">
+        <f>B$19*D36</f>
+        <v/>
+      </c>
+      <c r="D36" s="27" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Estimativa fica mais confiável a cada fatura completa anotada.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A26:B27">
+    <cfRule type="expression" priority="1" dxfId="2">
+      <formula>AND(ISNUMBER($B$26),$B$26&lt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Resumo da planilha em três blocos separados: fatura do cartão, vale e conta
A fatura do cartão (o que se paga) e o vale-alimentação (saldo da empresa)
não aparecem mais somados em nenhuma coluna, grade ou gráfico.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U9H2bpPTgH33XhYCozzWVS
</commit_message>
<xml_diff>
--- a/planilha/Gastos_Casa.xlsx
+++ b/planilha/Gastos_Casa.xlsx
@@ -57,12 +57,12 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="000000FF"/>
+      <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
+      <color rgb="000000FF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -82,7 +82,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -96,12 +96,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E3F1EA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E3F1EA"/>
+        <fgColor rgb="006B4599"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDE6F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003366A6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6EDF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDF0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -122,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -133,35 +158,49 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -175,6 +214,11 @@
           <fgColor rgb="00F8CBAD"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00BF1A1A"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -267,7 +311,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Cartão e conta por fatura (sai do bolso)</a:t>
+              <a:t>Fatura do cartão por período</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -282,7 +326,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Resumo'!B4</f>
+              <f>'Resumo'!C5</f>
             </strRef>
           </tx>
           <spPr>
@@ -292,36 +336,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Resumo'!$A$5:$A$16</f>
+              <f>'Resumo'!$A$6:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Resumo'!$B$5:$B$16</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Resumo'!D4</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Resumo'!$A$5:$A$16</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Resumo'!$D$5:$D$16</f>
+              <f>'Resumo'!$C$6:$C$17</f>
             </numRef>
           </val>
         </ser>
@@ -347,29 +367,11 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>R$</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -388,18 +390,24 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Por categoria na fatura atual (todas as formas)</a:t>
+              <a:t>Vale-alimentação: gasto e saldo por período</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
     </title>
     <plotArea>
-      <pieChart>
-        <varyColors val="1"/>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="stacked"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Resumo'!H5</f>
+            </strRef>
+          </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
@@ -407,20 +415,66 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Resumo'!$K$14:$K$19</f>
+              <f>'Resumo'!$A$6:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Resumo'!$L$14:$L$19</f>
+              <f>'Resumo'!$H$6:$H$17</f>
             </numRef>
           </val>
         </ser>
-        <dLbls>
-          <showPercent val="1"/>
-        </dLbls>
-        <firstSliceAng val="0"/>
-      </pieChart>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Resumo'!I5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Resumo'!$A$6:$A$17</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Resumo'!$I$6:$I$17</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="100"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
     </plotArea>
     <legend>
       <legendPos val="r"/>
@@ -516,7 +570,7 @@
     <author>Gastos Casa</author>
   </authors>
   <commentList>
-    <comment ref="A5" authorId="0" shapeId="0">
+    <comment ref="A6" authorId="0" shapeId="0">
       <text>
         <t>Início da primeira fatura anotada (26/10/2026, fechamento dos cartões). As seguintes são calculadas.</t>
       </text>
@@ -611,10 +665,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>30</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6480000" cy="2880000"/>
+    <ext cx="4680000" cy="2520000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -631,12 +685,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>6</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>30</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4320000" cy="2880000"/>
+    <ext cx="4680000" cy="2520000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1448,32 +1502,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W19"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="3" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="13" customWidth="1" min="19" max="19"/>
-    <col width="13" customWidth="1" min="20" max="20"/>
-    <col width="13" customWidth="1" min="21" max="21"/>
-    <col width="13" customWidth="1" min="22" max="22"/>
-    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="2" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="2" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="2" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1486,285 +1530,119 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cada fatura vai do dia 26 ao dia 25. Cartão = crédito (paga no mês seguinte); Vale = sai do saldo do vale; Conta = Pix, débito e dinheiro.</t>
+          <t>Cada bloco é um dinheiro diferente e não se soma com os outros. Cada período vai do dia 26 ao dia 25.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>Fatura (início)</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Cartão</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Vale</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Conta</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>FATURA DO CARTÃO DE CRÉDITO — o que vocês vão pagar</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>VALE-ALIMENTAÇÃO — saldo que a empresa coloca</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>CONTA — Pix, débito, dinheiro</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Cartão + conta (usado no Planejamento)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Início</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Fim</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Valor da fatura</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Compras no cartão</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Vs. fatura anterior</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>Crédito do vale</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>Gasto no vale</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>Saldo do vale</t>
+        </is>
+      </c>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>Gasto na conta</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>Cartão + conta</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>Gastos com valor</t>
-        </is>
-      </c>
-      <c r="G4" s="1" t="inlineStr">
-        <is>
-          <t>Sem valor</t>
-        </is>
-      </c>
-      <c r="H4" s="1" t="inlineStr">
-        <is>
-          <t>Cartão + conta vs. anterior</t>
-        </is>
-      </c>
-      <c r="I4" s="1" t="inlineStr">
-        <is>
-          <t>Gasto total da casa</t>
-        </is>
-      </c>
-      <c r="K4" s="7" t="inlineStr">
-        <is>
-          <t>Categoria</t>
-        </is>
-      </c>
-      <c r="L4" s="8">
-        <f>A5</f>
-        <v/>
-      </c>
-      <c r="M4" s="8">
-        <f>A6</f>
-        <v/>
-      </c>
-      <c r="N4" s="8">
-        <f>A7</f>
-        <v/>
-      </c>
-      <c r="O4" s="8">
-        <f>A8</f>
-        <v/>
-      </c>
-      <c r="P4" s="8">
-        <f>A9</f>
-        <v/>
-      </c>
-      <c r="Q4" s="8">
-        <f>A10</f>
-        <v/>
-      </c>
-      <c r="R4" s="8">
-        <f>A11</f>
-        <v/>
-      </c>
-      <c r="S4" s="8">
-        <f>A12</f>
-        <v/>
-      </c>
-      <c r="T4" s="8">
-        <f>A13</f>
-        <v/>
-      </c>
-      <c r="U4" s="8">
-        <f>A14</f>
-        <v/>
-      </c>
-      <c r="V4" s="8">
-        <f>A15</f>
-        <v/>
-      </c>
-      <c r="W4" s="8">
-        <f>A16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="n">
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="n">
         <v>46321</v>
       </c>
-      <c r="B5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
-        <v/>
-      </c>
-      <c r="C5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="D5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
-        <v/>
-      </c>
-      <c r="E5" s="5">
-        <f>B5+D5</f>
-        <v/>
-      </c>
-      <c r="F5" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="G5" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1),Lançamentos!$D$2:$D$1001,"")</f>
-        <v/>
-      </c>
-      <c r="H5" s="5" t="inlineStr"/>
-      <c r="I5" s="10">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A5,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A5,1))</f>
-        <v/>
-      </c>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
-          <t>Alimentação</t>
-        </is>
-      </c>
-      <c r="L5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
-        <v/>
-      </c>
-      <c r="M5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
-        <v/>
-      </c>
-      <c r="N5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
-        <v/>
-      </c>
-      <c r="O5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
-        <v/>
-      </c>
-      <c r="P5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
-        <v/>
-      </c>
-      <c r="Q5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
-        <v/>
-      </c>
-      <c r="R5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
-        <v/>
-      </c>
-      <c r="S5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
-        <v/>
-      </c>
-      <c r="T5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;T$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(T$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
-        <v/>
-      </c>
-      <c r="U5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;U$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(U$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
-        <v/>
-      </c>
-      <c r="V5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;V$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(V$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
-        <v/>
-      </c>
-      <c r="W5" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;W$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(W$4,1),Lançamentos!$C$2:$C$1001,$K5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3">
-        <f>EDATE(A5,1)</f>
-        <v/>
-      </c>
-      <c r="B6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
-        <v/>
-      </c>
-      <c r="C6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="D6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
-        <v/>
-      </c>
-      <c r="E6" s="5">
-        <f>B6+D6</f>
-        <v/>
-      </c>
-      <c r="F6" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="G6" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1),Lançamentos!$D$2:$D$1001,"")</f>
+      <c r="B6" s="3">
+        <f>EDATE(A6,1)-1</f>
+        <v/>
+      </c>
+      <c r="C6" s="14">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B6,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="D6" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B6,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="G6" s="5">
+        <f>IF($A6&gt;Planejamento!$B$6,"",Planejamento!$B$22)</f>
         <v/>
       </c>
       <c r="H6" s="5">
-        <f>IF(E6=0,"",E6-E5)</f>
-        <v/>
-      </c>
-      <c r="I6" s="10">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A6,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A6,1))</f>
-        <v/>
-      </c>
-      <c r="K6" s="11" t="inlineStr">
-        <is>
-          <t>Casa/contas</t>
-        </is>
-      </c>
-      <c r="L6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B6,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="I6" s="14">
+        <f>IF(G6="","",G6-H6)</f>
+        <v/>
+      </c>
+      <c r="K6" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B6,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B6,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B6,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
         <v/>
       </c>
       <c r="M6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
-        <v/>
-      </c>
-      <c r="N6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
-        <v/>
-      </c>
-      <c r="O6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
-        <v/>
-      </c>
-      <c r="P6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
-        <v/>
-      </c>
-      <c r="Q6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
-        <v/>
-      </c>
-      <c r="R6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
-        <v/>
-      </c>
-      <c r="S6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
-        <v/>
-      </c>
-      <c r="T6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;T$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(T$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
-        <v/>
-      </c>
-      <c r="U6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;U$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(U$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
-        <v/>
-      </c>
-      <c r="V6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;V$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(V$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
-        <v/>
-      </c>
-      <c r="W6" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;W$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(W$4,1),Lançamentos!$C$2:$C$1001,$K6)</f>
+        <f>C6+K6</f>
         <v/>
       </c>
     </row>
@@ -1773,89 +1651,40 @@
         <f>EDATE(A6,1)</f>
         <v/>
       </c>
-      <c r="B7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
-        <v/>
-      </c>
-      <c r="C7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="D7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+      <c r="B7" s="3">
+        <f>EDATE(A7,1)-1</f>
+        <v/>
+      </c>
+      <c r="C7" s="14">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A7,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B7,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="D7" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A7,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B7,Lançamentos!$E$2:$E$1001,"Crédito")</f>
         <v/>
       </c>
       <c r="E7" s="5">
-        <f>B7+D7</f>
-        <v/>
-      </c>
-      <c r="F7" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="G7" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <f>IF(C7=0,"",C7-C6)</f>
+        <v/>
+      </c>
+      <c r="G7" s="5">
+        <f>IF($A7&gt;Planejamento!$B$6,"",Planejamento!$B$22)</f>
         <v/>
       </c>
       <c r="H7" s="5">
-        <f>IF(E7=0,"",E7-E6)</f>
-        <v/>
-      </c>
-      <c r="I7" s="10">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A7,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A7,1))</f>
-        <v/>
-      </c>
-      <c r="K7" s="11" t="inlineStr">
-        <is>
-          <t>Transporte</t>
-        </is>
-      </c>
-      <c r="L7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A7,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B7,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="I7" s="14">
+        <f>IF(G7="","",G7-H7)</f>
+        <v/>
+      </c>
+      <c r="K7" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A7,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B7,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A7,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B7,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A7,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B7,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
         <v/>
       </c>
       <c r="M7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
-        <v/>
-      </c>
-      <c r="N7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
-        <v/>
-      </c>
-      <c r="O7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
-        <v/>
-      </c>
-      <c r="P7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
-        <v/>
-      </c>
-      <c r="Q7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
-        <v/>
-      </c>
-      <c r="R7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
-        <v/>
-      </c>
-      <c r="S7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
-        <v/>
-      </c>
-      <c r="T7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;T$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(T$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
-        <v/>
-      </c>
-      <c r="U7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;U$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(U$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
-        <v/>
-      </c>
-      <c r="V7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;V$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(V$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
-        <v/>
-      </c>
-      <c r="W7" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;W$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(W$4,1),Lançamentos!$C$2:$C$1001,$K7)</f>
+        <f>C7+K7</f>
         <v/>
       </c>
     </row>
@@ -1864,89 +1693,40 @@
         <f>EDATE(A7,1)</f>
         <v/>
       </c>
-      <c r="B8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
-        <v/>
-      </c>
-      <c r="C8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="D8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+      <c r="B8" s="3">
+        <f>EDATE(A8,1)-1</f>
+        <v/>
+      </c>
+      <c r="C8" s="14">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A8,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B8,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="D8" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A8,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B8,Lançamentos!$E$2:$E$1001,"Crédito")</f>
         <v/>
       </c>
       <c r="E8" s="5">
-        <f>B8+D8</f>
-        <v/>
-      </c>
-      <c r="F8" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="G8" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <f>IF(C8=0,"",C8-C7)</f>
+        <v/>
+      </c>
+      <c r="G8" s="5">
+        <f>IF($A8&gt;Planejamento!$B$6,"",Planejamento!$B$22)</f>
         <v/>
       </c>
       <c r="H8" s="5">
-        <f>IF(E8=0,"",E8-E7)</f>
-        <v/>
-      </c>
-      <c r="I8" s="10">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A8,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A8,1))</f>
-        <v/>
-      </c>
-      <c r="K8" s="11" t="inlineStr">
-        <is>
-          <t>Saúde</t>
-        </is>
-      </c>
-      <c r="L8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A8,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B8,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="I8" s="14">
+        <f>IF(G8="","",G8-H8)</f>
+        <v/>
+      </c>
+      <c r="K8" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A8,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B8,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A8,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B8,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A8,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B8,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
         <v/>
       </c>
       <c r="M8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
-        <v/>
-      </c>
-      <c r="N8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
-        <v/>
-      </c>
-      <c r="O8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
-        <v/>
-      </c>
-      <c r="P8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
-        <v/>
-      </c>
-      <c r="Q8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
-        <v/>
-      </c>
-      <c r="R8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
-        <v/>
-      </c>
-      <c r="S8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
-        <v/>
-      </c>
-      <c r="T8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;T$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(T$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
-        <v/>
-      </c>
-      <c r="U8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;U$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(U$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
-        <v/>
-      </c>
-      <c r="V8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;V$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(V$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
-        <v/>
-      </c>
-      <c r="W8" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;W$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(W$4,1),Lançamentos!$C$2:$C$1001,$K8)</f>
+        <f>C8+K8</f>
         <v/>
       </c>
     </row>
@@ -1955,89 +1735,40 @@
         <f>EDATE(A8,1)</f>
         <v/>
       </c>
-      <c r="B9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
-        <v/>
-      </c>
-      <c r="C9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="D9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+      <c r="B9" s="3">
+        <f>EDATE(A9,1)-1</f>
+        <v/>
+      </c>
+      <c r="C9" s="14">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A9,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B9,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="D9" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A9,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B9,Lançamentos!$E$2:$E$1001,"Crédito")</f>
         <v/>
       </c>
       <c r="E9" s="5">
-        <f>B9+D9</f>
-        <v/>
-      </c>
-      <c r="F9" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="G9" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <f>IF(C9=0,"",C9-C8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="5">
+        <f>IF($A9&gt;Planejamento!$B$6,"",Planejamento!$B$22)</f>
         <v/>
       </c>
       <c r="H9" s="5">
-        <f>IF(E9=0,"",E9-E8)</f>
-        <v/>
-      </c>
-      <c r="I9" s="10">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A9,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A9,1))</f>
-        <v/>
-      </c>
-      <c r="K9" s="11" t="inlineStr">
-        <is>
-          <t>Lazer</t>
-        </is>
-      </c>
-      <c r="L9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A9,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B9,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="I9" s="14">
+        <f>IF(G9="","",G9-H9)</f>
+        <v/>
+      </c>
+      <c r="K9" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A9,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B9,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A9,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B9,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A9,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B9,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
         <v/>
       </c>
       <c r="M9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
-        <v/>
-      </c>
-      <c r="N9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
-        <v/>
-      </c>
-      <c r="O9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
-        <v/>
-      </c>
-      <c r="P9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
-        <v/>
-      </c>
-      <c r="Q9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
-        <v/>
-      </c>
-      <c r="R9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
-        <v/>
-      </c>
-      <c r="S9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
-        <v/>
-      </c>
-      <c r="T9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;T$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(T$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
-        <v/>
-      </c>
-      <c r="U9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;U$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(U$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
-        <v/>
-      </c>
-      <c r="V9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;V$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(V$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
-        <v/>
-      </c>
-      <c r="W9" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;W$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(W$4,1),Lançamentos!$C$2:$C$1001,$K9)</f>
+        <f>C9+K9</f>
         <v/>
       </c>
     </row>
@@ -2046,89 +1777,40 @@
         <f>EDATE(A9,1)</f>
         <v/>
       </c>
-      <c r="B10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
-        <v/>
-      </c>
-      <c r="C10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="D10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+      <c r="B10" s="3">
+        <f>EDATE(A10,1)-1</f>
+        <v/>
+      </c>
+      <c r="C10" s="14">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A10,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B10,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="D10" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A10,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B10,Lançamentos!$E$2:$E$1001,"Crédito")</f>
         <v/>
       </c>
       <c r="E10" s="5">
-        <f>B10+D10</f>
-        <v/>
-      </c>
-      <c r="F10" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="G10" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <f>IF(C10=0,"",C10-C9)</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>IF($A10&gt;Planejamento!$B$6,"",Planejamento!$B$22)</f>
         <v/>
       </c>
       <c r="H10" s="5">
-        <f>IF(E10=0,"",E10-E9)</f>
-        <v/>
-      </c>
-      <c r="I10" s="10">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A10,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A10,1))</f>
-        <v/>
-      </c>
-      <c r="K10" s="11" t="inlineStr">
-        <is>
-          <t>Outros</t>
-        </is>
-      </c>
-      <c r="L10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;L$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(L$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A10,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B10,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="I10" s="14">
+        <f>IF(G10="","",G10-H10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A10,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B10,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A10,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B10,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A10,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B10,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
         <v/>
       </c>
       <c r="M10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;M$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(M$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
-        <v/>
-      </c>
-      <c r="N10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;N$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(N$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
-        <v/>
-      </c>
-      <c r="O10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;O$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(O$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
-        <v/>
-      </c>
-      <c r="P10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;P$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(P$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
-        <v/>
-      </c>
-      <c r="Q10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Q$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(Q$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
-        <v/>
-      </c>
-      <c r="R10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;R$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(R$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
-        <v/>
-      </c>
-      <c r="S10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;S$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(S$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
-        <v/>
-      </c>
-      <c r="T10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;T$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(T$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
-        <v/>
-      </c>
-      <c r="U10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;U$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(U$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
-        <v/>
-      </c>
-      <c r="V10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;V$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(V$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
-        <v/>
-      </c>
-      <c r="W10" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;W$4,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(W$4,1),Lançamentos!$C$2:$C$1001,$K10)</f>
+        <f>C10+K10</f>
         <v/>
       </c>
     </row>
@@ -2137,89 +1819,40 @@
         <f>EDATE(A10,1)</f>
         <v/>
       </c>
-      <c r="B11" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
-        <v/>
-      </c>
-      <c r="C11" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="D11" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+      <c r="B11" s="3">
+        <f>EDATE(A11,1)-1</f>
+        <v/>
+      </c>
+      <c r="C11" s="14">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A11,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B11,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="D11" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A11,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B11,Lançamentos!$E$2:$E$1001,"Crédito")</f>
         <v/>
       </c>
       <c r="E11" s="5">
-        <f>B11+D11</f>
-        <v/>
-      </c>
-      <c r="F11" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="G11" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <f>IF(C11=0,"",C11-C10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="5">
+        <f>IF($A11&gt;Planejamento!$B$6,"",Planejamento!$B$22)</f>
         <v/>
       </c>
       <c r="H11" s="5">
-        <f>IF(E11=0,"",E11-E10)</f>
-        <v/>
-      </c>
-      <c r="I11" s="10">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A11,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A11,1))</f>
-        <v/>
-      </c>
-      <c r="K11" s="12" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="L11" s="13">
-        <f>SUM(L5:L10)</f>
-        <v/>
-      </c>
-      <c r="M11" s="13">
-        <f>SUM(M5:M10)</f>
-        <v/>
-      </c>
-      <c r="N11" s="13">
-        <f>SUM(N5:N10)</f>
-        <v/>
-      </c>
-      <c r="O11" s="13">
-        <f>SUM(O5:O10)</f>
-        <v/>
-      </c>
-      <c r="P11" s="13">
-        <f>SUM(P5:P10)</f>
-        <v/>
-      </c>
-      <c r="Q11" s="13">
-        <f>SUM(Q5:Q10)</f>
-        <v/>
-      </c>
-      <c r="R11" s="13">
-        <f>SUM(R5:R10)</f>
-        <v/>
-      </c>
-      <c r="S11" s="13">
-        <f>SUM(S5:S10)</f>
-        <v/>
-      </c>
-      <c r="T11" s="13">
-        <f>SUM(T5:T10)</f>
-        <v/>
-      </c>
-      <c r="U11" s="13">
-        <f>SUM(U5:U10)</f>
-        <v/>
-      </c>
-      <c r="V11" s="13">
-        <f>SUM(V5:V10)</f>
-        <v/>
-      </c>
-      <c r="W11" s="13">
-        <f>SUM(W5:W10)</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A11,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B11,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="I11" s="14">
+        <f>IF(G11="","",G11-H11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A11,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B11,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A11,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B11,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A11,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B11,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="M11" s="5">
+        <f>C11+K11</f>
         <v/>
       </c>
     </row>
@@ -2228,36 +1861,40 @@
         <f>EDATE(A11,1)</f>
         <v/>
       </c>
-      <c r="B12" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
-        <v/>
-      </c>
-      <c r="C12" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="D12" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+      <c r="B12" s="3">
+        <f>EDATE(A12,1)-1</f>
+        <v/>
+      </c>
+      <c r="C12" s="14">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A12,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B12,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="D12" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A12,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B12,Lançamentos!$E$2:$E$1001,"Crédito")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>B12+D12</f>
-        <v/>
-      </c>
-      <c r="F12" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="G12" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <f>IF(C12=0,"",C12-C11)</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>IF($A12&gt;Planejamento!$B$6,"",Planejamento!$B$22)</f>
         <v/>
       </c>
       <c r="H12" s="5">
-        <f>IF(E12=0,"",E12-E11)</f>
-        <v/>
-      </c>
-      <c r="I12" s="10">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A12,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A12,1))</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A12,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B12,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="I12" s="14">
+        <f>IF(G12="","",G12-H12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A12,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B12,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A12,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B12,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A12,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B12,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="M12" s="5">
+        <f>C12+K12</f>
         <v/>
       </c>
     </row>
@@ -2266,45 +1903,40 @@
         <f>EDATE(A12,1)</f>
         <v/>
       </c>
-      <c r="B13" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
-        <v/>
-      </c>
-      <c r="C13" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="D13" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+      <c r="B13" s="3">
+        <f>EDATE(A13,1)-1</f>
+        <v/>
+      </c>
+      <c r="C13" s="14">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A13,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B13,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="D13" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A13,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B13,Lançamentos!$E$2:$E$1001,"Crédito")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>B13+D13</f>
-        <v/>
-      </c>
-      <c r="F13" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="G13" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <f>IF(C13=0,"",C13-C12)</f>
+        <v/>
+      </c>
+      <c r="G13" s="5">
+        <f>IF($A13&gt;Planejamento!$B$6,"",Planejamento!$B$22)</f>
         <v/>
       </c>
       <c r="H13" s="5">
-        <f>IF(E13=0,"",E13-E12)</f>
-        <v/>
-      </c>
-      <c r="I13" s="10">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A13,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A13,1))</f>
-        <v/>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>Fatura atual</t>
-        </is>
-      </c>
-      <c r="L13" s="14">
-        <f>Planejamento!$B$6</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A13,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B13,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="I13" s="14">
+        <f>IF(G13="","",G13-H13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A13,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B13,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A13,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B13,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A13,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B13,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="M13" s="5">
+        <f>C13+K13</f>
         <v/>
       </c>
     </row>
@@ -2313,44 +1945,40 @@
         <f>EDATE(A13,1)</f>
         <v/>
       </c>
-      <c r="B14" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
-        <v/>
-      </c>
-      <c r="C14" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="D14" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+      <c r="B14" s="3">
+        <f>EDATE(A14,1)-1</f>
+        <v/>
+      </c>
+      <c r="C14" s="14">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A14,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B14,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="D14" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A14,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B14,Lançamentos!$E$2:$E$1001,"Crédito")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>B14+D14</f>
-        <v/>
-      </c>
-      <c r="F14" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="G14" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <f>IF(C14=0,"",C14-C13)</f>
+        <v/>
+      </c>
+      <c r="G14" s="5">
+        <f>IF($A14&gt;Planejamento!$B$6,"",Planejamento!$B$22)</f>
         <v/>
       </c>
       <c r="H14" s="5">
-        <f>IF(E14=0,"",E14-E13)</f>
-        <v/>
-      </c>
-      <c r="I14" s="10">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A14,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A14,1))</f>
-        <v/>
-      </c>
-      <c r="K14" s="11">
-        <f>K5</f>
-        <v/>
-      </c>
-      <c r="L14" s="15">
-        <f>INDEX($L5:$W5,MATCH($L$13,$L$4:$W$4,0))</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A14,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B14,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="I14" s="14">
+        <f>IF(G14="","",G14-H14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A14,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B14,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A14,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B14,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A14,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B14,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="M14" s="5">
+        <f>C14+K14</f>
         <v/>
       </c>
     </row>
@@ -2359,44 +1987,40 @@
         <f>EDATE(A14,1)</f>
         <v/>
       </c>
-      <c r="B15" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
-        <v/>
-      </c>
-      <c r="C15" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="D15" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+      <c r="B15" s="3">
+        <f>EDATE(A15,1)-1</f>
+        <v/>
+      </c>
+      <c r="C15" s="14">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A15,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B15,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="D15" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A15,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B15,Lançamentos!$E$2:$E$1001,"Crédito")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>B15+D15</f>
-        <v/>
-      </c>
-      <c r="F15" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="G15" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <f>IF(C15=0,"",C15-C14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="5">
+        <f>IF($A15&gt;Planejamento!$B$6,"",Planejamento!$B$22)</f>
         <v/>
       </c>
       <c r="H15" s="5">
-        <f>IF(E15=0,"",E15-E14)</f>
-        <v/>
-      </c>
-      <c r="I15" s="10">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A15,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A15,1))</f>
-        <v/>
-      </c>
-      <c r="K15" s="11">
-        <f>K6</f>
-        <v/>
-      </c>
-      <c r="L15" s="15">
-        <f>INDEX($L6:$W6,MATCH($L$13,$L$4:$W$4,0))</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A15,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B15,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="I15" s="14">
+        <f>IF(G15="","",G15-H15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A15,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B15,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A15,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B15,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A15,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B15,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="M15" s="5">
+        <f>C15+K15</f>
         <v/>
       </c>
     </row>
@@ -2405,78 +2029,264 @@
         <f>EDATE(A15,1)</f>
         <v/>
       </c>
-      <c r="B16" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$E$2:$E$1001,"Crédito")</f>
-        <v/>
-      </c>
-      <c r="C16" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
-        <v/>
-      </c>
-      <c r="D16" s="5">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+      <c r="B16" s="3">
+        <f>EDATE(A16,1)-1</f>
+        <v/>
+      </c>
+      <c r="C16" s="14">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A16,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B16,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="D16" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A16,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B16,Lançamentos!$E$2:$E$1001,"Crédito")</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>B16+D16</f>
-        <v/>
-      </c>
-      <c r="F16" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$D$2:$D$1001,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="G16" s="4">
-        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1),Lançamentos!$D$2:$D$1001,"")</f>
+        <f>IF(C16=0,"",C16-C15)</f>
+        <v/>
+      </c>
+      <c r="G16" s="5">
+        <f>IF($A16&gt;Planejamento!$B$6,"",Planejamento!$B$22)</f>
         <v/>
       </c>
       <c r="H16" s="5">
-        <f>IF(E16=0,"",E16-E15)</f>
-        <v/>
-      </c>
-      <c r="I16" s="10">
-        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;A16,Lançamentos!$A$2:$A$1001,"&lt;"&amp;EDATE(A16,1))</f>
-        <v/>
-      </c>
-      <c r="K16" s="11">
-        <f>K7</f>
-        <v/>
-      </c>
-      <c r="L16" s="15">
-        <f>INDEX($L7:$W7,MATCH($L$13,$L$4:$W$4,0))</f>
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A16,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B16,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="I16" s="14">
+        <f>IF(G16="","",G16-H16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A16,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B16,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A16,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B16,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A16,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B16,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="M16" s="5">
+        <f>C16+K16</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="K17" s="11">
-        <f>K8</f>
-        <v/>
-      </c>
-      <c r="L17" s="15">
-        <f>INDEX($L8:$W8,MATCH($L$13,$L$4:$W$4,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="K18" s="11">
-        <f>K9</f>
-        <v/>
-      </c>
-      <c r="L18" s="15">
-        <f>INDEX($L9:$W9,MATCH($L$13,$L$4:$W$4,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="K19" s="11">
-        <f>K10</f>
-        <v/>
-      </c>
-      <c r="L19" s="15">
-        <f>INDEX($L10:$W10,MATCH($L$13,$L$4:$W$4,0))</f>
-        <v/>
+      <c r="A17" s="3">
+        <f>EDATE(A16,1)</f>
+        <v/>
+      </c>
+      <c r="B17" s="3">
+        <f>EDATE(A17,1)-1</f>
+        <v/>
+      </c>
+      <c r="C17" s="14">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A17,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B17,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="D17" s="4">
+        <f>COUNTIFS(Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A17,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B17,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="E17" s="5">
+        <f>IF(C17=0,"",C17-C16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="5">
+        <f>IF($A17&gt;Planejamento!$B$6,"",Planejamento!$B$22)</f>
+        <v/>
+      </c>
+      <c r="H17" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A17,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B17,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="I17" s="14">
+        <f>IF(G17="","",G17-H17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A17,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B17,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A17,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B17,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;$A17,Lançamentos!$A$2:$A$1001,"&lt;="&amp;$B17,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+      <c r="M17" s="5">
+        <f>C17+K17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Fatura atual por categoria (cada coluna é um dinheiro diferente)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Vale</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Conta</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="B22" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A22,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C22" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A22,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D22" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A22,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A22,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A22,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Casa/contas</t>
+        </is>
+      </c>
+      <c r="B23" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A23,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C23" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A23,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D23" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A23,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A23,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A23,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Transporte</t>
+        </is>
+      </c>
+      <c r="B24" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A24,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C24" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A24,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D24" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A24,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A24,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A24,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="B25" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A25,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C25" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A25,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D25" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A25,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A25,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A25,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Lazer</t>
+        </is>
+      </c>
+      <c r="B26" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A26,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C26" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A26,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D26" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A26,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A26,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A26,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="B27" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A27,Lançamentos!$E$2:$E$1001,"Crédito")</f>
+        <v/>
+      </c>
+      <c r="C27" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A27,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
+        <v/>
+      </c>
+      <c r="D27" s="5">
+        <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A27,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A27,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;Planejamento!$B$6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;Planejamento!$B$7,Lançamentos!$C$2:$C$1001,$A27,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B28" s="14">
+        <f>SUM(B22:B27)</f>
+        <v/>
+      </c>
+      <c r="C28" s="14">
+        <f>SUM(C22:C27)</f>
+        <v/>
+      </c>
+      <c r="D28" s="14">
+        <f>SUM(D22:D27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Não some as colunas: o cartão vai para a fatura, o vale sai do saldo do vale e a conta sai do banco.</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="A4:E4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="I6:I17">
+    <cfRule type="expression" priority="1" dxfId="2">
+      <formula>AND(ISNUMBER(I6),I6&lt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -2514,59 +2324,59 @@
       </c>
     </row>
     <row r="3">
-      <c r="E3" s="16" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Gastos fixos mensais fora do grupo</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Margem de segurança</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="22" t="n">
         <v>0.1</v>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="23" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="23" t="inlineStr">
         <is>
           <t>Valor por mês</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Dia de fechamento da fatura</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
+      <c r="B5" s="24" t="n">
         <v>26</v>
       </c>
-      <c r="E5" s="20" t="n"/>
-      <c r="F5" s="21" t="n"/>
+      <c r="E5" s="25" t="n"/>
+      <c r="F5" s="26" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Fatura atual (início)</t>
         </is>
       </c>
       <c r="B6" s="3">
-        <f>IF(COUNT(Lançamentos!$A$2:$A$1001)=0,Resumo!$A$5,DATE(YEAR(MAX(Lançamentos!$A$2:$A$1001)),MONTH(MAX(Lançamentos!$A$2:$A$1001))-IF(DAY(MAX(Lançamentos!$A$2:$A$1001))&lt;B5,1,0),B5))</f>
-        <v/>
-      </c>
-      <c r="E6" s="20" t="n"/>
-      <c r="F6" s="21" t="n"/>
+        <f>IF(COUNT(Lançamentos!$A$2:$A$1001)=0,Resumo!$A$6,DATE(YEAR(MAX(Lançamentos!$A$2:$A$1001)),MONTH(MAX(Lançamentos!$A$2:$A$1001))-IF(DAY(MAX(Lançamentos!$A$2:$A$1001))&lt;B5,1,0),B5))</f>
+        <v/>
+      </c>
+      <c r="E6" s="25" t="n"/>
+      <c r="F6" s="26" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Fatura atual (fim)</t>
         </is>
@@ -2575,46 +2385,46 @@
         <f>EDATE(B6,1)-1</f>
         <v/>
       </c>
-      <c r="E7" s="20" t="n"/>
-      <c r="F7" s="21" t="n"/>
+      <c r="E7" s="25" t="n"/>
+      <c r="F7" s="26" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Dias na fatura</t>
         </is>
       </c>
-      <c r="B8" s="22">
+      <c r="B8" s="27">
         <f>B7-B6+1</f>
         <v/>
       </c>
-      <c r="E8" s="20" t="n"/>
-      <c r="F8" s="21" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="26" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Dias com anotações</t>
         </is>
       </c>
-      <c r="B9" s="22">
+      <c r="B9" s="27">
         <f>IF(COUNT(Lançamentos!$A$2:$A$1001)=0,0,MAX(Lançamentos!$A$2:$A$1001)-B6+1)</f>
         <v/>
       </c>
-      <c r="E9" s="20" t="n"/>
-      <c r="F9" s="21" t="n"/>
+      <c r="E9" s="25" t="n"/>
+      <c r="F9" s="26" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Fatura do cartão + conta (sai do bolso)</t>
         </is>
       </c>
-      <c r="E10" s="20" t="n"/>
-      <c r="F10" s="21" t="n"/>
+      <c r="E10" s="25" t="n"/>
+      <c r="F10" s="26" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Cartão (crédito) nesta fatura</t>
         </is>
@@ -2623,11 +2433,11 @@
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B7,Lançamentos!$E$2:$E$1001,"Crédito")</f>
         <v/>
       </c>
-      <c r="E11" s="20" t="n"/>
-      <c r="F11" s="21" t="n"/>
+      <c r="E11" s="25" t="n"/>
+      <c r="F11" s="26" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>Conta (Pix, débito, dinheiro)</t>
         </is>
@@ -2636,11 +2446,11 @@
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B7,Lançamentos!$E$2:$E$1001,"Pix")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B7,Lançamentos!$E$2:$E$1001,"Débito")+SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B7,Lançamentos!$E$2:$E$1001,"Dinheiro")</f>
         <v/>
       </c>
-      <c r="E12" s="20" t="n"/>
-      <c r="F12" s="21" t="n"/>
+      <c r="E12" s="25" t="n"/>
+      <c r="F12" s="26" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Cartão + conta</t>
         </is>
@@ -2649,11 +2459,11 @@
         <f>B11+B12</f>
         <v/>
       </c>
-      <c r="E13" s="20" t="n"/>
-      <c r="F13" s="21" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="26" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>Média por dia</t>
         </is>
@@ -2662,11 +2472,11 @@
         <f>IF(B9=0,0,B13/B9)</f>
         <v/>
       </c>
-      <c r="E14" s="20" t="n"/>
-      <c r="F14" s="21" t="n"/>
+      <c r="E14" s="25" t="n"/>
+      <c r="F14" s="26" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Projeção até o dia 25</t>
         </is>
@@ -2675,37 +2485,37 @@
         <f>B13+B14*(B8-B9)</f>
         <v/>
       </c>
-      <c r="E15" s="20" t="n"/>
-      <c r="F15" s="21" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="26" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Faturas anteriores usadas</t>
         </is>
       </c>
-      <c r="B16" s="22">
-        <f>COUNTIFS(Resumo!$A$5:$A$16,"&gt;="&amp;EDATE(B6,-3),Resumo!$A$5:$A$16,"&lt;"&amp;B6,Resumo!$E$5:$E$16,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="E16" s="20" t="n"/>
-      <c r="F16" s="21" t="n"/>
+      <c r="B16" s="27">
+        <f>COUNTIFS(Resumo!$A$6:$A$17,"&gt;="&amp;EDATE(B6,-3),Resumo!$A$6:$A$17,"&lt;"&amp;B6,Resumo!$M$6:$M$17,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="E16" s="25" t="n"/>
+      <c r="F16" s="26" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>Média por fatura (cartão + conta)</t>
         </is>
       </c>
       <c r="B17" s="5">
-        <f>IF(B16=0,B15,AVERAGEIFS(Resumo!$E$5:$E$16,Resumo!$A$5:$A$16,"&gt;="&amp;EDATE(B6,-3),Resumo!$A$5:$A$16,"&lt;"&amp;B6,Resumo!$E$5:$E$16,"&gt;0"))</f>
-        <v/>
-      </c>
-      <c r="E17" s="20" t="n"/>
-      <c r="F17" s="21" t="n"/>
+        <f>IF(B16=0,B15,AVERAGEIFS(Resumo!$M$6:$M$17,Resumo!$A$6:$A$17,"&gt;="&amp;EDATE(B6,-3),Resumo!$A$6:$A$17,"&lt;"&amp;B6,Resumo!$M$6:$M$17,"&gt;0"))</f>
+        <v/>
+      </c>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="26" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>Gastos fixos fora do grupo</t>
         </is>
@@ -2714,49 +2524,49 @@
         <f>SUM(F5:F24)</f>
         <v/>
       </c>
-      <c r="E18" s="20" t="n"/>
-      <c r="F18" s="21" t="n"/>
+      <c r="E18" s="25" t="n"/>
+      <c r="F18" s="26" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="inlineStr">
+      <c r="A19" s="28" t="inlineStr">
         <is>
           <t>Separar por fatura</t>
         </is>
       </c>
-      <c r="B19" s="24">
+      <c r="B19" s="29">
         <f>(B17+B18)*(1+B4)</f>
         <v/>
       </c>
-      <c r="E19" s="20" t="n"/>
-      <c r="F19" s="21" t="n"/>
+      <c r="E19" s="25" t="n"/>
+      <c r="F19" s="26" t="n"/>
     </row>
     <row r="20">
-      <c r="E20" s="20" t="n"/>
-      <c r="F20" s="21" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="26" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>Vale-alimentação (sai do saldo do vale)</t>
         </is>
       </c>
-      <c r="E21" s="20" t="n"/>
-      <c r="F21" s="21" t="n"/>
+      <c r="E21" s="25" t="n"/>
+      <c r="F21" s="26" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="A22" s="21" t="inlineStr">
         <is>
           <t>Vale por mês</t>
         </is>
       </c>
-      <c r="B22" s="25" t="n">
+      <c r="B22" s="30" t="n">
         <v>2643.77</v>
       </c>
-      <c r="E22" s="20" t="n"/>
-      <c r="F22" s="21" t="n"/>
+      <c r="E22" s="25" t="n"/>
+      <c r="F22" s="26" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>Gasto no vale nesta fatura</t>
         </is>
@@ -2765,11 +2575,11 @@
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B7,Lançamentos!$E$2:$E$1001,"Vale-alimentação")</f>
         <v/>
       </c>
-      <c r="E23" s="20" t="n"/>
-      <c r="F23" s="21" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="26" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="A24" s="21" t="inlineStr">
         <is>
           <t>Saldo atual do vale</t>
         </is>
@@ -2778,11 +2588,11 @@
         <f>IF(B22="","Preencha o valor do vale",B22-B23)</f>
         <v/>
       </c>
-      <c r="E24" s="20" t="n"/>
-      <c r="F24" s="21" t="n"/>
+      <c r="E24" s="25" t="n"/>
+      <c r="F24" s="26" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>Média por dia no vale</t>
         </is>
@@ -2798,7 +2608,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="21" t="inlineStr">
         <is>
           <t>Saldo projetado no dia 25</t>
         </is>
@@ -2809,12 +2619,12 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>Situação do vale</t>
         </is>
       </c>
-      <c r="B27" s="26">
+      <c r="B27" s="31">
         <f>IF(B22="","",IF(B26&lt;0,"Atenção: no ritmo atual o vale acaba antes do dia 25; faltam cerca de R$ "&amp;ROUND(-B26,0)&amp;", que vão cair no cartão ou na conta.","Dentro do saldo do vale"))</f>
         <v/>
       </c>
@@ -2825,13 +2635,13 @@
           <t>Gasto total da casa nesta fatura (referência)</t>
         </is>
       </c>
-      <c r="B29" s="10">
+      <c r="B29" s="32">
         <f>SUMIFS(Lançamentos!$D$2:$D$1001,Lançamentos!$A$2:$A$1001,"&gt;="&amp;B6,Lançamentos!$A$2:$A$1001,"&lt;="&amp;B7)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>Reserva por horizonte (cartão + conta)</t>
         </is>
@@ -2855,7 +2665,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="inlineStr">
+      <c r="A33" s="21" t="inlineStr">
         <is>
           <t>1 fatura</t>
         </is>
@@ -2868,12 +2678,12 @@
         <f>B$19*D33</f>
         <v/>
       </c>
-      <c r="D33" s="27" t="n">
+      <c r="D33" s="33" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="inlineStr">
+      <c r="A34" s="21" t="inlineStr">
         <is>
           <t>3 faturas</t>
         </is>
@@ -2886,12 +2696,12 @@
         <f>B$19*D34</f>
         <v/>
       </c>
-      <c r="D34" s="27" t="n">
+      <c r="D34" s="33" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="inlineStr">
+      <c r="A35" s="21" t="inlineStr">
         <is>
           <t>6 faturas</t>
         </is>
@@ -2904,12 +2714,12 @@
         <f>B$19*D35</f>
         <v/>
       </c>
-      <c r="D35" s="27" t="n">
+      <c r="D35" s="33" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="inlineStr">
+      <c r="A36" s="21" t="inlineStr">
         <is>
           <t>12 faturas</t>
         </is>
@@ -2922,7 +2732,7 @@
         <f>B$19*D36</f>
         <v/>
       </c>
-      <c r="D36" s="27" t="n">
+      <c r="D36" s="33" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2935,7 +2745,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A26:B27">
-    <cfRule type="expression" priority="1" dxfId="2">
+    <cfRule type="expression" priority="1" dxfId="3">
       <formula>AND(ISNUMBER($B$26),$B$26&lt;0)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Importar conversa até 28/10; parcelamento (Nx) e fatura atual pela data de hoje
- Parser divide compras parceladas em lançamentos mensais (centavos na
  última parcela), ignora <Mensagem editada> e aceita "valor - credito".
- Compra no vale sem pista de categoria vira Alimentação.
- Painel e planilha passam a usar a data de hoje para a fatura atual, para
  que parcelas futuras não mudem a fatura em análise.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U9H2bpPTgH33XhYCozzWVS
</commit_message>
<xml_diff>
--- a/planilha/Gastos_Casa.xlsx
+++ b/planilha/Gastos_Casa.xlsx
@@ -21,9 +21,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="&quot;R$&quot; #,##0.00;-&quot;R$&quot; #,##0.00;&quot;-&quot;"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="166" formatCode="&quot;R$&quot; #,##0.00;-&quot;R$&quot; #,##0.00;&quot;-&quot;"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -153,9 +153,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -175,8 +175,8 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -188,13 +188,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1024,7 +1024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1073,124 +1073,424 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n"/>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
+      <c r="A2" s="3" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Lasanha feira</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Bruna</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n"/>
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
+      <c r="A3" s="3" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Bolo banana + fatia focaccia feira</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Bruna</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
+      <c r="A4" s="3" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Cafe manha brasco</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Vale-alimentação</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Bruna</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
+      <c r="A5" s="3" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Padaria</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>14.52</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Tassio</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
+      <c r="A6" s="3" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Zaffari</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>73.20999999999999</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Vale-alimentação</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Tassio</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="n"/>
+      <c r="A7" s="3" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>2 tênis (parcela 1/6)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Tassio</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
+      <c r="A8" s="3" t="n">
+        <v>46354</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>2 tênis (parcela 2/6)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Tassio</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="n"/>
+      <c r="A9" s="3" t="n">
+        <v>46384</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2 tênis (parcela 3/6)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Tassio</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
+      <c r="A10" s="3" t="n">
+        <v>46415</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>2 tênis (parcela 4/6)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Tassio</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
+      <c r="A11" s="3" t="n">
+        <v>46446</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>2 tênis (parcela 5/6)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Tassio</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="n"/>
+      <c r="A12" s="3" t="n">
+        <v>46474</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>2 tênis (parcela 6/6)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>33.35</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Tassio</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n"/>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
+      <c r="A13" s="3" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Center shopping</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>53.96</v>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Vale-alimentação</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Tassio</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n"/>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="n"/>
+      <c r="A14" s="3" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Presente colega trabalho</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Tassio</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n"/>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
+      <c r="A15" s="3" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Paulinho frutas</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Bruna</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="n"/>
+      <c r="A16" s="3" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Masssagem</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Lazer</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Bruna</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
@@ -1471,6 +1771,126 @@
       <c r="D51" s="5" t="n"/>
       <c r="E51" s="4" t="n"/>
       <c r="F51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="n"/>
+      <c r="B52" s="4" t="n"/>
+      <c r="C52" s="4" t="n"/>
+      <c r="D52" s="5" t="n"/>
+      <c r="E52" s="4" t="n"/>
+      <c r="F52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="4" t="n"/>
+      <c r="D53" s="5" t="n"/>
+      <c r="E53" s="4" t="n"/>
+      <c r="F53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="4" t="n"/>
+      <c r="C54" s="4" t="n"/>
+      <c r="D54" s="5" t="n"/>
+      <c r="E54" s="4" t="n"/>
+      <c r="F54" s="4" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="4" t="n"/>
+      <c r="C55" s="4" t="n"/>
+      <c r="D55" s="5" t="n"/>
+      <c r="E55" s="4" t="n"/>
+      <c r="F55" s="4" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="n"/>
+      <c r="B56" s="4" t="n"/>
+      <c r="C56" s="4" t="n"/>
+      <c r="D56" s="5" t="n"/>
+      <c r="E56" s="4" t="n"/>
+      <c r="F56" s="4" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="n"/>
+      <c r="B57" s="4" t="n"/>
+      <c r="C57" s="4" t="n"/>
+      <c r="D57" s="5" t="n"/>
+      <c r="E57" s="4" t="n"/>
+      <c r="F57" s="4" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="n"/>
+      <c r="B58" s="4" t="n"/>
+      <c r="C58" s="4" t="n"/>
+      <c r="D58" s="5" t="n"/>
+      <c r="E58" s="4" t="n"/>
+      <c r="F58" s="4" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="n"/>
+      <c r="B59" s="4" t="n"/>
+      <c r="C59" s="4" t="n"/>
+      <c r="D59" s="5" t="n"/>
+      <c r="E59" s="4" t="n"/>
+      <c r="F59" s="4" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="n"/>
+      <c r="B60" s="4" t="n"/>
+      <c r="C60" s="4" t="n"/>
+      <c r="D60" s="5" t="n"/>
+      <c r="E60" s="4" t="n"/>
+      <c r="F60" s="4" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="n"/>
+      <c r="B61" s="4" t="n"/>
+      <c r="C61" s="4" t="n"/>
+      <c r="D61" s="5" t="n"/>
+      <c r="E61" s="4" t="n"/>
+      <c r="F61" s="4" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="n"/>
+      <c r="B62" s="4" t="n"/>
+      <c r="C62" s="4" t="n"/>
+      <c r="D62" s="5" t="n"/>
+      <c r="E62" s="4" t="n"/>
+      <c r="F62" s="4" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="n"/>
+      <c r="B63" s="4" t="n"/>
+      <c r="C63" s="4" t="n"/>
+      <c r="D63" s="5" t="n"/>
+      <c r="E63" s="4" t="n"/>
+      <c r="F63" s="4" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="n"/>
+      <c r="B64" s="4" t="n"/>
+      <c r="C64" s="4" t="n"/>
+      <c r="D64" s="5" t="n"/>
+      <c r="E64" s="4" t="n"/>
+      <c r="F64" s="4" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="n"/>
+      <c r="B65" s="4" t="n"/>
+      <c r="C65" s="4" t="n"/>
+      <c r="D65" s="5" t="n"/>
+      <c r="E65" s="4" t="n"/>
+      <c r="F65" s="4" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="n"/>
+      <c r="B66" s="4" t="n"/>
+      <c r="C66" s="4" t="n"/>
+      <c r="D66" s="5" t="n"/>
+      <c r="E66" s="4" t="n"/>
+      <c r="F66" s="4" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1001"/>

</xml_diff>

<commit_message>
Gerador: fatura atual pela data de hoje
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U9H2bpPTgH33XhYCozzWVS
</commit_message>
<xml_diff>
--- a/planilha/Gastos_Casa.xlsx
+++ b/planilha/Gastos_Casa.xlsx
@@ -597,12 +597,12 @@
     </comment>
     <comment ref="B6" authorId="0" shapeId="0">
       <text>
-        <t>Fatura do gasto mais recente.</t>
+        <t>Fatura que contém a data de hoje.</t>
       </text>
     </comment>
     <comment ref="B9" authorId="0" shapeId="0">
       <text>
-        <t>Do dia 26 até o gasto mais recente.</t>
+        <t>Do dia 26 até hoje.</t>
       </text>
     </comment>
     <comment ref="B11" authorId="0" shapeId="0">
@@ -2785,11 +2785,11 @@
     <row r="6">
       <c r="A6" s="21" t="inlineStr">
         <is>
-          <t>Fatura atual (início)</t>
+          <t>Fatura atual (início) — pela data de hoje</t>
         </is>
       </c>
       <c r="B6" s="3">
-        <f>IF(COUNT(Lançamentos!$A$2:$A$1001)=0,Resumo!$A$6,DATE(YEAR(MAX(Lançamentos!$A$2:$A$1001)),MONTH(MAX(Lançamentos!$A$2:$A$1001))-IF(DAY(MAX(Lançamentos!$A$2:$A$1001))&lt;B5,1,0),B5))</f>
+        <f>DATE(YEAR(TODAY()),MONTH(TODAY())-IF(DAY(TODAY())&lt;B5,1,0),B5)</f>
         <v/>
       </c>
       <c r="E6" s="25" t="n"/>
@@ -2824,11 +2824,11 @@
     <row r="9">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>Dias com anotações</t>
+          <t>Dias já passados na fatura</t>
         </is>
       </c>
       <c r="B9" s="27">
-        <f>IF(COUNT(Lançamentos!$A$2:$A$1001)=0,0,MAX(Lançamentos!$A$2:$A$1001)-B6+1)</f>
+        <f>MAX(0,MIN(TODAY(),B7)-B6+1)</f>
         <v/>
       </c>
       <c r="E9" s="25" t="n"/>

</xml_diff>